<commit_message>
设计侧登记批（2026-09-02）：UPG-68 DEL manifest 补（红线23）；UPG-43a/69 拆卡派单；E4 archived 档；UPG-24 作废+26 验收+04/45 补合段
</commit_message>
<xml_diff>
--- a/工单系统/工单表.xlsx
+++ b/工单系统/工单表.xlsx
@@ -446,7 +446,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I59"/>
+  <dimension ref="A1:I60"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -672,12 +672,12 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>✅ 验收通过（并入 UPG-02 合并单验收）｜ 设计师/方案设计/UPG-04_Obsidian工具包_方案设计.md</t>
+          <t>✅ 验收通过（并入 UPG-02 合并单验收）｜ 设计师/方案设计/UPG-04_Obsidian工具包_方案设计.md→ 已合 main@</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>合 main@2026-08-29（merge 8a205d6 已推 origin）**；原</t>
+          <t>已合 main@2026-08-29（merge 8a205d6 已推 origin；随 UPG-02 合并单｜obsidian.* 工具面</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
@@ -1320,7 +1320,7 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>📌 **重排 @2026-09-02（用户拍板：App 内浏览器先 MCP 改造）**｜本卡=**43a App 侧 WebMCP Hub</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
@@ -1837,7 +1837,7 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>✅**规范文档已交付 @2026-08-29**（`设计师/方案设计/MOV设计规范_v1.md`，待用户过目）</t>
+          <t>❌ **已作废 @2026-09-02**（用户拍板：设计规范 v1 文档已删｜由 v2/v2.1+UPG-50 外观组件体系接替；本卡销账</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
@@ -1941,12 +1941,12 @@
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>✅ 验收通过（用户确认「已实现」）@2026-09-02（feat/sidebar-brand 7a6dff6+0fdfe87：品牌区 lo</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>合 main</t>
+          <t>**分支未合 main（162 分叉）｜待设计师合 main**）</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
@@ -2087,7 +2087,7 @@
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>**待设计师合 main → 审验员**</t>
+          <t>**已合 main @2026-08-31 → 审验员**（approval 体系随 UPG-58/62/63 合入；ApprovalSer</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
@@ -3158,12 +3158,13 @@
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>📌 施工中（P0·3~5 工作日；CT-13/14 契约后补不阻塞）  **v3 定稿 @2026-09-01（二轮大神 9.1/10 可</t>
+          <t>📌 施工中（P0·3~5 工作日；CT-13/14 契约后补不阻塞）+ → 方案 v3 定稿 @2026-09-01（二轮大神 9.1/1</t>
         </is>
       </c>
       <c r="F59" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>✅ R1 复验带缺陷通过 @2026-09-01（feat/upg68 35b0008｜HIGH/M1/M2 三缺口 security_re</t>
         </is>
       </c>
       <c r="G59" t="inlineStr">
@@ -3177,6 +3178,53 @@
         </is>
       </c>
       <c r="I59" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>UPG-69</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>WebMCP 站点试点（mow.kim 工单站「站点=业务工具」第一站）</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>📌 新立 @2026-09-02（用户拍板：App 内浏览器先 MCP 改造｜站点侧并行试点）｜待派单可认领</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G60" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H60" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I60" t="inlineStr">
         <is>
           <t>—</t>
         </is>

</xml_diff>

<commit_message>
回炉 Failed to fetch 根治：server 加 CORS（ACAO */OPTIONS 预检 204/允许 Content-Type）——file:// 双击打开页面也能成功 POST；测试残留已清
</commit_message>
<xml_diff>
--- a/工单系统/工单表.xlsx
+++ b/工单系统/工单表.xlsx
@@ -845,27 +845,27 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>P1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>✅ 方案完成｜ feat/upg08 → main aa09882（ff，含R1/R2修复+同步）</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>✅C R2 修复完成</t>
+          <t>修复完成，待</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>验收员✅全部通过 @2026-08-26（R1 复验 P1×3 全消 + R2 消 P3，无遗留缺陷）</t>
+          <t>🔨 打回修复派单，待程序员领修复（优先原施工者 C；撞单按认领规则）｜ 验收缺陷明细见 `0027-mov\docs\ACCEPTANCE</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>**设计师✅已合 main @2026-08-26**（`aa09882`，ff 合入，同步产物 json 已移出版本库）</t>
+          <t>已合 main的单基于最新 main 重开分支）；再认领：工单表第 9 行备注追加 `认领: &lt;agent&gt; R1修复 @&lt;时间&gt;`； 2.</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">

</xml_diff>

<commit_message>
BoardWriteEngine 组件化落地（Hono+zod+薄壳，大神 v2 定稿）：①依赖 hono 4.13.5+@hono/node-server 2.1.1+zod 4.5.4（registry tgz 手装）②board-server v3 迁 Hono（/api/board/v1: health/capabilities/card.reject/restore/move；Origin+随机 WriteToken 守卫；11 错误码；兼容 CORS+OPTIONS）③board-engine 薄壳（状态迁移矩阵/单写锁/审计 Ledger/事务-备份→改库→sync→回滚）④前端 BoardAPI（Token 获取/Idempotency-Key/成功局部更新行不整页 reload/离线提示）⑤端到端全链实测（UNAUTHORIZED/CONFLICT/reject/restore/Ledger/并发锁）+修复 UPG-08 旧残留
</commit_message>
<xml_diff>
--- a/工单系统/工单表.xlsx
+++ b/工单系统/工单表.xlsx
@@ -845,27 +845,27 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>P1</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>✅ 方案完成｜ feat/upg08 → main aa09882（ff，含R1/R2修复+同步）</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>修复完成，待</t>
+          <t>✅C R2 修复完成</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>🔨 打回修复派单，待程序员领修复（优先原施工者 C；撞单按认领规则）｜ 验收缺陷明细见 `0027-mov\docs\ACCEPTANCE</t>
+          <t>验收员✅全部通过 @2026-08-26（R1 复验 P1×3 全消 + R2 消 P3，无遗留缺陷）</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>已合 main的单基于最新 main 重开分支）；再认领：工单表第 9 行备注追加 `认领: &lt;agent&gt; R1修复 @&lt;时间&gt;`； 2.</t>
+          <t>**设计师✅已合 main @2026-08-26**（`aa09882`，ff 合入，同步产物 json 已移出版本库）</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">

</xml_diff>

<commit_message>
UPG-103 已认领：Claude CLI 2.1.150（mov-upg103 @cfa7d607）
</commit_message>
<xml_diff>
--- a/工单系统/工单表.xlsx
+++ b/工单系统/工单表.xlsx
@@ -4714,17 +4714,17 @@
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>P1</t>
+          <t>P1 → 🆕 **已认领 @2026-09-04 20:50**</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>📌 **已派单·待认领 @2026-09-04**（拆分主线批④/共 8 批｜串行纪律：批③ cfa7d607 已合，本批基=main 顶</t>
+          <t>📌 **已派单·待认领 @2026-09-04**</t>
         </is>
       </c>
       <c r="E91" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>🆕 **已认领 @2026-09-04 20:50**（程序员/Claude-kimi，worktree mov-upg103，branc</t>
         </is>
       </c>
       <c r="F91" t="inlineStr">

</xml_diff>

<commit_message>
UPG-103 合 main 登记 @97d7ca31：审验员转通过+设计师合入+verify-hash 终态 HASH_OK
</commit_message>
<xml_diff>
--- a/工单系统/工单表.xlsx
+++ b/工单系统/工单表.xlsx
@@ -4724,12 +4724,12 @@
       </c>
       <c r="F91" t="inlineStr">
         <is>
-          <t>⚠️ **审验 unresolved @2026-09-05**（实质可信｜审验员独立复现 recon103 9/9 块 ALL_OK；**</t>
+          <t>✅ **审验员转通过 @2026-09-05**（四断收口逐项复核全绿：STD v2 重冻=51584a7d 一致/DEL 绑定 manif</t>
         </is>
       </c>
       <c r="G91" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>✅ **设计师合 main @97d7ca31**（2026-09-05：批④ chips/胶囊面搬移全链合入；合后 verify-hash</t>
         </is>
       </c>
       <c r="H91" t="inlineStr">
@@ -4855,7 +4855,7 @@
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>📋 **架构评审稿已出**：`人体载体/数字人体_融入MOV架构_评审稿_2026-09-05.md`（与 MOV 契合度审查+合规红线+</t>
+          <t>✅ **大神评审通过 8.8/10（有条件）@2026-09-05 → v2.1 冻结稿已出**：`人体载体/数字人体_融入MOV架构_评审</t>
         </is>
       </c>
       <c r="E94" t="inlineStr">

</xml_diff>

<commit_message>
UPG-107 交付：DELIVERY_UPG107_2026-09-05.md（八步全过+3 锚亲杀+真机 5 场景）+ manifest（DEL-UPG107-20260905-001 code=31640fc8 审验 ok:true）+ UPG107-evidence 5 份——feat/upg107 31640fc8 待验收；coverage PARTIAL 设计师裁决位（记忆页 UI 可视化留接缝）
</commit_message>
<xml_diff>
--- a/工单系统/工单表.xlsx
+++ b/工单系统/工单表.xlsx
@@ -446,7 +446,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I94"/>
+  <dimension ref="A1:I95"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2928,12 +2928,12 @@
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>】；【⛔ **部分打回 @2026-08-31**（ACCEPTANCE_LOG 9e764fb）：feat/upg63 0580fa8 基</t>
+          <t>⚠️ **错挂注记 @2026-09-05（设计师）**：以下打回段主体=feat/upg63 0580fa8，属 **UPG-63** 卡</t>
         </is>
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>合 main</t>
+          <t>✅ **已合 main @34c37f54（补登 @2026-09-05，设计师核物）**：=交付提交 e4aa2a6 的 patch-id</t>
         </is>
       </c>
       <c r="H54" t="inlineStr">
@@ -4881,6 +4881,53 @@
       <c r="I94" t="inlineStr">
         <is>
           <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>UPG-107</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>Memory OS 类型化 payload（Semantic 池子结构化演进）</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="D95" t="inlineStr">
+        <is>
+          <t>裁决位]；DEL-UPG107-20260905-001[code=31640fc8/artifact=fc07ee63/manifest=</t>
+        </is>
+      </c>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>✅**C 完成 @2026-09-05**（feat/upg107 **31640fc8** 已 push origin[origin=gi</t>
+        </is>
+      </c>
+      <c r="F95" t="inlineStr">
+        <is>
+          <t>审验ok:true]/报告=程序员/交付报告/DELIVERY_UPG107_2026-09-05.md｜状态区投影锚+交付段详）</t>
+        </is>
+      </c>
+      <c r="G95" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H95" t="inlineStr">
+        <is>
+          <t>设计师/方案设计/04_记忆/Memory_OS_类型化payload_设计_v1_2026-09-05.md</t>
+        </is>
+      </c>
+      <c r="I95" t="inlineStr">
+        <is>
+          <t>DEL-UPG107-20260905-001</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
UPG-69 收口：STD 补冻+DEL 绑定（MANIFEST_OK）+两表+合 main @44a414ae 登记+§P59 W6 行补
</commit_message>
<xml_diff>
--- a/工单系统/工单表.xlsx
+++ b/工单系统/工单表.xlsx
@@ -446,7 +446,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I97"/>
+  <dimension ref="A1:I106"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1258,22 +1258,22 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>UPG-14</t>
+          <t>W-09</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>设置页收口（账号卡接真 + 退出登录去重 + 两行死链修复）</t>
+          <t>资产档案表（T6 落地：商标/证书/域名/密钥登记收编）</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>P1</t>
+          <t>P2</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>方案完成待派单（P2）</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
@@ -1283,12 +1283,12 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>✅验收员通过 @2026-08-28（R2 e16fae8 三判据全过 + R2 复修 04341d2 全产物口径零命中）</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>**设计师✅已合 main @2026-08-28**（全链 9323975→ce5ab0d→e16fae8→1825338→04341d2</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
@@ -1305,22 +1305,22 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>UPG-15</t>
+          <t>W-10</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>登录页死锁修（登录钮常可点 + 协议整行可点）</t>
+          <t>事件日历视图 + 总览仪表盘四组件</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>P1</t>
+          <t>P2</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>方案完成待派单（P2）</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
@@ -1330,12 +1330,12 @@
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>✅验收员通过 @2026-08-28（151fdb1 独立复核：L1 全量 246 绿 + 变异亲杀 3/3 + L2 五图证据链；无缺陷）</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>**设计师✅已合 main @2026-08-28**（merge 509ab0c，ACCEPTANCE_LOG append-only 冲</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
@@ -1352,12 +1352,12 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>UPG-16</t>
+          <t>UPG-14</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>release 签名配置收口（明文口令外移）</t>
+          <t>设置页收口（账号卡接真 + 退出登录去重 + 两行死链修复）</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -1377,12 +1377,12 @@
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>✅验收员通过 @2026-08-28（172e67d 独立复核：L1 全量 243 绿 + apksigner 签名有效 + L2 口令文件</t>
+          <t>✅验收员通过 @2026-08-28（R2 e16fae8 三判据全过 + R2 复修 04341d2 全产物口径零命中）</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>**设计师✅已合 main @2026-08-28**（merge ee312f5，已推 origin；主 worktree 签名参数已落</t>
+          <t>**设计师✅已合 main @2026-08-28**（全链 9323975→ce5ab0d→e16fae8→1825338→04341d2</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
@@ -1399,12 +1399,12 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>UPG-17</t>
+          <t>UPG-15</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>App demo 假数据全清（Vue 侧）</t>
+          <t>登录页死锁修（登录钮常可点 + 协议整行可点）</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -1419,17 +1419,17 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>C 完成@2026-08-28（feat/upg17 96c963d，3 commits：926d70b feat+1f532cb buil</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>✅**验收员通过 @2026-08-28 深夜**（独立复核全过：L1 `--rerun-tasks` 36 类 253/0/0 吻合+sy</t>
+          <t>✅验收员通过 @2026-08-28（151fdb1 独立复核：L1 全量 246 绿 + 变异亲杀 3/3 + L2 五图证据链；无缺陷）</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>✅**设计师已合 main @2026-08-28（merge 36d7f6e 已推 origin）｜UPG-17 全链闭环**（合后全量</t>
+          <t>**设计师✅已合 main @2026-08-28**（merge 509ab0c，ACCEPTANCE_LOG append-only 冲</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
@@ -1446,37 +1446,37 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>UPG-18</t>
+          <t>UPG-16</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Android 死代码清理</t>
+          <t>release 签名配置收口（明文口令外移）</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>P2</t>
+          <t>P1</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>✅ 方案完成</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>🛠 在施 C @2026-08-30 01:39（认领=worktree mov-upg18 branch feat/upg18）</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>✅ **验收通过 @2026-08-30**（ACCEPTANCE_LOG「验收：UPG-18 死代码清理」段：L1 全量 376/0/0</t>
+          <t>✅验收员通过 @2026-08-28（172e67d 独立复核：L1 全量 243 绿 + apksigner 签名有效 + L2 口令文件</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>✅ **已合 main @2026-08-30**（merge **6103bb8c**｜批1-4+批2修正全量在链；resolve：Mai</t>
+          <t>**设计师✅已合 main @2026-08-28**（merge ee312f5，已推 origin；主 worktree 签名参数已落</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
@@ -1493,12 +1493,12 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>UPG-19</t>
+          <t>UPG-17</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>应用图标换 MOV 竖眼 Logo</t>
+          <t>App demo 假数据全清（Vue 侧）</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -1513,17 +1513,17 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>C 完成@2026-08-28（feat/upg17 96c963d，3 commits：926d70b feat+1f532cb buil</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>✅**验收员复验通过 @2026-08-28**（验收对象=入库链 feat/upg19 fa8fdd1+2c6b777+82a5322：L</t>
+          <t>✅**验收员通过 @2026-08-28 深夜**（独立复核全过：L1 `--rerun-tasks` 36 类 253/0/0 吻合+sy</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>**设计师✅已合 main @2026-08-28**（merge 17b4e04 已推 origin；mov-upg19 worktree</t>
+          <t>✅**设计师已合 main @2026-08-28（merge 36d7f6e 已推 origin）｜UPG-17 全链闭环**（合后全量</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
@@ -1540,37 +1540,37 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>UPG-20</t>
+          <t>UPG-18</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>聊天页 chips 改造 v2（气泡式 切换模型+MCP 工具）</t>
+          <t>Android 死代码清理</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>P1</t>
+          <t>P2</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>**转派 @2026-08-28 18:35（用户拍板）**：C 认领后零提交 11h（分支仍 8aaa999）、主线在 UPG-17｜转派</t>
+          <t>✅ 方案完成</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>🔨 已派单，C 已认领在施 @2026-08-28 07:45（worktree=mov-upg20 branch=feat/upg20，</t>
+          <t>🛠 在施 C @2026-08-30 01:39（认领=worktree mov-upg18 branch feat/upg18）</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>✅验收员复验通过 @2026-08-28 深夜（装机实证：二级 refit 重锚底部 2062≤chip 顶 2113 贴上沿不悬空、MCP</t>
+          <t>✅ **验收通过 @2026-08-30**（ACCEPTANCE_LOG「验收：UPG-18 死代码清理」段：L1 全量 376/0/0</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>✅**设计师已合 main @2026-08-28（merge 974f33a 已推 origin）｜UPG-20 全链闭环**（合前独立复</t>
+          <t>✅ **已合 main @2026-08-30**（merge **6103bb8c**｜批1-4+批2修正全量在链；resolve：Mai</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
@@ -1587,12 +1587,12 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>UPG-21</t>
+          <t>W-11</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>聊天页输入框回车键=发送（IME 发送键修复）</t>
+          <t>account-service 安全加固</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -1607,17 +1607,17 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>✅程序员 C 完成 @2026-08-29（feat/upg21 a14ee64，基于 main 198e26f；报告 DELIVERY_U</t>
+          <t>✅ C 完成 @2026-09-05（655b148d，9 隐患清零，待验收）</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>验收员通过 @2026-08-29（</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>✅**已合 main @2026-08-29（merge 5170421 已推 origin）｜UPG-21 全链闭环**（审验员五步独立实</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
@@ -1627,19 +1627,19 @@
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>DEL-W11-20260905-001</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>UPG-22</t>
+          <t>S-04</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>记忆尾单（UPG-05 遗留收口：COVER_HIT 装配打点 + 剧本断言 + 冗余清理）</t>
+          <t>MOV 域迁移（市场迁 mov-ai.cn，API 双跑兜底）</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -1649,27 +1649,27 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>方案完成待派单（ICP 硬阻塞注记：09-04 备案号已上页脚，阻塞或已解除待核实）</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>✅**C 完成 @2026-08-29 16:48**（feat/upg22 **aacb15b** 已 push origin，基线已 f</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>✅**验收员 R1 L2 复验通过 @2026-08-29**（三连全过：①装配打点落新 session jsonl memory/ref</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>✅**已合 main @2026-08-29**（程序员代行设计师：rebase 87787b8 后 ff-only **495060f**</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>设计师/派单/UPG-22_记忆尾单_派单_2026-08-29.md</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
@@ -1681,12 +1681,12 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>UPG-23</t>
+          <t>S-05</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>本地 tab「本机能力总览」+ 主页钉选小按钮</t>
+          <t>市场首页去 demo 化（接 registry + 空态诚实 + 死链清理）</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -1701,17 +1701,17 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>修复完成@2026-08-29**（feat/upg23 **0bfa4fa** 已 push origin；`runOnUiThread</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>✅**验收员复验通过 @2026-08-29**（diff 恰 1 行无夹带 + L1 338/0/0 亲跑 + 真机 5556：钉选/取消</t>
+          <t>✅ 验收通过 @2026-08-29（公网+服务器双实证）</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>✅**审验通过 → 已合 main @2026-08-29**（查验员逐项亲核确认；设计师 §六抽查：R1_05 主页钉选排免重启当场可见亲</t>
+          <t>✅ 已闭环（服务端生效，无 main 合并对象）</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
@@ -1728,12 +1728,12 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>UPG-24</t>
+          <t>S-06</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>MOV 设计规范 v1（风格定性 + token 坐标表）</t>
+          <t>市场站 bug 批修 + 死文件清理</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -1743,12 +1743,12 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>❌ **已作废 @2026-09-02**（用户拍板：设计规范 v1 文档已删｜由 v2/v2.1+UPG-50 外观组件体系接替；本卡销账</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>✅ 程序员完成 @2026-08-29（87ec0a1；部署卡腾讯云扫码墙）</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
@@ -1763,7 +1763,7 @@
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>设计师/方案设计/MOV设计规范_v1.md</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I29" t="inlineStr">
@@ -1775,42 +1775,42 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>UPG-25</t>
+          <t>W-12</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>UI 瑕疵批修（规范 v1 待并轨清单 13 项）</t>
+          <t>workbench 前端小修批</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>P1</t>
+          <t>P3</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>裁决=MainActivity/PhotoAskSheet 文本底色取 UiTokens、primary 保 upg40 mov_prima</t>
+          <t>方案完成待派单（P3 小修批）</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>C 完成@2026-08-29**（feat/upg25 **62986c2** 已推 origin｜含 merge origin/main</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>❌**打回@2026-08-30**：与已合 UPG-40 换肤**同文件双改**（WorkbenchPage/demo.js/MainAc</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>✅**已合 main @2026-08-30**（设计师 merge 8f8debd，含 2ccce25；§六 抽查通过 13 项+候选C</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>设计师/派单/UPG-25_重修_派单_2026-08-30.md</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I30" t="inlineStr">
@@ -1822,12 +1822,12 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>UPG-26</t>
+          <t>S-07</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>侧边栏品牌区换 logo+黑字 + 抽屉展开占比 61.8%</t>
+          <t>MOV 公众官网一期（用户下载门户 + 创作者开发者中心）</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -1837,7 +1837,7 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>裁决]；用户确认已实现 @2026-09-02）→</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
@@ -1847,12 +1847,12 @@
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>✅ 验收通过（用户确认「已实现」）@2026-09-02（feat/sidebar-brand 7a6dff6+0fdfe87：品牌区 lo</t>
+          <t>✅ 验收通过 @2026-08-28</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>**分支未合 main（162 分叉）｜已合 main@2026-09-02（feat/sidebar-brand 7a6dff6/0fdf</t>
+          <t>✅ 已合 main @ce1ab567</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
@@ -1869,12 +1869,12 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>UPG-28</t>
+          <t>UPG-19</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>obsidian.file.write 审批闸修复（isHarmless file.write 特判误捕）</t>
+          <t>应用图标换 MOV 竖眼 Logo</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
@@ -1884,27 +1884,27 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>✅**方案 v1 已出 @2026-08-29**（`设计师/方案设计/UPG-28_obsidian写入审批闸修复_方案设计.md`）</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>✅**程序员 C 完成 @2026-08-30 01:05**（feat/upg28 **443b288** 已 push origin，基</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>✅**验收员验收通过 @2026-08-30**（L1 377/0/0 亲跑+变异 M1/M2 双锚亲杀+L2 采纳模拟器证据[真机 ASK</t>
+          <t>✅**验收员复验通过 @2026-08-28**（验收对象=入库链 feat/upg19 fa8fdd1+2c6b777+82a5322：L</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>✅**已合 main @443b288**（ff-only 已推 origin，合后全量复跑 377/0/0 绿；worktree mov-</t>
+          <t>**设计师✅已合 main @2026-08-28**（merge 17b4e04 已推 origin；mov-upg19 worktree</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>设计师/方案设计/UPG-28_obsidian写入审批闸修复_方案设计.md</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I32" t="inlineStr">
@@ -1916,12 +1916,12 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>UPG-44</t>
+          <t>S-08</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>AcceptanceJudge B1 观察层（UPG-06 批2 剩项）</t>
+          <t>官网「能力市场」页（/home/market/，与 App 市场同源）</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
@@ -1931,27 +1931,27 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>裁决criteria+AI 回复→verdict/失败静默]；**投影剔键硬红**=Surface.deriveEventMessage 显</t>
+          <t>**转派 @2026-08-28 18:35（用户拍板）**：C 认领后零提交 11h（分支仍 8aaa999）、主线在 UPG-17｜转派</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>C 完成@2026-08-30 04:05**（feat/upg44 **122945b** 基底 main 3263f10 已 push；</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>审验通过 → 已合 main @2026-08-30**（设计师 §六抽查 + rebase 后 ff-only **801b8fc 已推</t>
+          <t>✅ 验收通过 @2026-08-28（471ae65 独立复核）</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>✅**验收+审验通过 → 已合 main @2026-08-30**（设计师 §六抽查 + rebase 后 ff-only **801b8</t>
+          <t>✅ 已合 main @dc1405bc</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>设计师/派单/UPG-44_AcceptanceJudge_B1_派单_2026-08-30.md</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I33" t="inlineStr">
@@ -1963,42 +1963,42 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>UPG-45</t>
+          <t>UPG-20</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>审批 · Approval Capability Registry（权限能力注册表）</t>
+          <t>聊天页 chips 改造 v2（气泡式 切换模型+MCP 工具）</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>P0</t>
+          <t>P1</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>🔨**已派单 @2026-08-30**（用户已转派；派单文本 `设计师/派单/UPG-45_审批_ApprovalRegistry_派单</t>
+          <t>**转派 @2026-08-28 18:35（用户拍板）**：C 认领后零提交 11h（分支仍 8aaa999）、主线在 UPG-17｜转派</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>🔨 已派单，C 已认领在施 @2026-08-28 07:45（worktree=mov-upg20 branch=feat/upg20，</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>✅**验收员通过 @2026-08-30**（ACCEPTANCE_LOG UPG-45，commit edf86d9）：核物[54行=as</t>
+          <t>✅验收员复验通过 @2026-08-28 深夜（装机实证：二级 refit 重锚底部 2062≤chip 顶 2113 贴上沿不悬空、MCP</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>**已合 main @2026-08-31 → 审验员**（approval 体系随 UPG-58/62/63 合入；ApprovalSer</t>
+          <t>✅**设计师已合 main @2026-08-28（merge 974f33a 已推 origin）｜UPG-20 全链闭环**（合前独立复</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>设计师\方案设计\审批弹窗_用户授权层_设计_v3_2026-08-30.md</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I34" t="inlineStr">
@@ -2010,42 +2010,42 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>UPG-46</t>
+          <t>UPG-21</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>工具联动 Runtime 契约（Tool Orchestration）</t>
+          <t>聊天页输入框回车键=发送（IME 发送键修复）</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>P0</t>
+          <t>P1</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>🔄 **用户拍板转交 @2026-09-05 02:19**（原认领程序员 Claude/wmw0027 做不了，用户指令转交）</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>✅**C 完成 @2026-09-05 03:02**（程序员 Kimi/kimi-cli，feat/upg46 **a8043aad**</t>
+          <t>✅程序员 C 完成 @2026-08-29（feat/upg21 a14ee64，基于 main 198e26f；报告 DELIVERY_U</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>✅ **验收员复验通过 @2026-09-05**（§P57 落档：六件核物全在/M-cycle 锚链成立/837 差 1 双方 P3 注记</t>
+          <t>验收员通过 @2026-08-29（</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>✅ **审验员确认+设计师合 main @7ccf0446**（2026-09-05：段①核心契约全链合入；段②=UPG-104） **卡点</t>
+          <t>✅**已合 main @2026-08-29（merge 5170421 已推 origin）｜UPG-21 全链闭环**（审验员五步独立实</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>设计师/派单/UPG-46_工具联动Runtime契约_派单_2026-09-02.md</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I35" t="inlineStr">
@@ -2057,42 +2057,42 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>UPG-47</t>
+          <t>UPG-22</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>主页胶囊系统（pin_type+stableId / 三区 / ＋管理弹层 / 点击分派 / 长按 / 第三态 / 气泡字数）</t>
+          <t>记忆尾单（UPG-05 遗留收口：COVER_HIT 装配打点 + 剧本断言 + 冗余清理）</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>P0</t>
+          <t>P1</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>🔨已派单</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>✅C 交付 @2026-08-30（feat/capsule-system **767228c+32ba01c** push；报告 程序员/</t>
+          <t>✅**C 完成 @2026-08-29 16:48**（feat/upg22 **aacb15b** 已 push origin，基线已 f</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>✅ **验收员复验 通过 @2026-09-04**（ACCEPTANCE_LOG §P54：4e5a2f7c 隔离 worktree[申报</t>
+          <t>✅**验收员 R1 L2 复验通过 @2026-08-29**（三连全过：①装配打点落新 session jsonl memory/ref</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>✅后续美化已合 main @2026-08-31（dock 对齐 **afc1ccd**：＋号圆形·随胶囊横滑·气泡左对齐胶囊；管理面板设置</t>
+          <t>✅**已合 main @2026-08-29**（程序员代行设计师：rebase 87787b8 后 ff-only **495060f**</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>设计师/派单/UPG-22_记忆尾单_派单_2026-08-29.md</t>
         </is>
       </c>
       <c r="I36" t="inlineStr">
@@ -2104,37 +2104,37 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>UPG-48</t>
+          <t>UPG-23</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Memory API 工程契约（记忆页:memory-core/memory-api 模块化）</t>
+          <t>本地 tab「本机能力总览」+ 主页钉选小按钮</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>P0</t>
+          <t>P1</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>🔨已派单 @2026-08-30</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>修复完成@2026-08-29**（feat/upg23 **0bfa4fa** 已 push origin；`runOnUiThread</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>❌**审验打回@2026-08-30（P1 边界违例）**｜MainActivity:582-598 直引 com.hermes.mov.m</t>
+          <t>✅**验收员复验通过 @2026-08-29**（diff 恰 1 行无夹带 + L1 338/0/0 亲跑 + 真机 5556：钉选/取消</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>✅**已合 main @2026-08-30**（设计师 merge 92d4c22[含 0aa0c07]，审验五步复核通过：零直触core</t>
+          <t>✅**审验通过 → 已合 main @2026-08-29**（查验员逐项亲核确认；设计师 §六抽查：R1_05 主页钉选排免重启当场可见亲</t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
@@ -2151,106 +2151,106 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>UPG-49</t>
+          <t>UPG-24</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>记忆页「我的记忆」UI 分层管理</t>
+          <t>MOV 设计规范 v1（风格定性 + token 坐标表）</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>P2</t>
+          <t>P1</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>✅ 方案 v4 定稿（记忆页分层管理_设计_v4 大神 9.2 冻结）</t>
+          <t>❌ **已作废 @2026-09-02**（用户拍板：设计规范 v1 文档已删｜由 v2/v2.1+UPG-50 外观组件体系接替；本卡销账</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>🔨 **程序员 R2 修复交付 @2026-09-01**（feat/upg49-r2 **5640bce** 已 push origin</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>✅ **审验通过 @2026-09-01**（integrity_review=confirmed：P2-1a 72px 像素实证+删📌</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>✅ **设计师终审合流 @2026-09-02**（B9edcc4 落档+工单库补登；2 治理项裁决见下）</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>设计师/方案设计/MOV设计规范_v1.md</t>
         </is>
       </c>
       <c r="I38" t="inlineStr">
         <is>
-          <t>DEL-UPG49-20260901-002</t>
+          <t>—</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>UPG-50</t>
+          <t>UPG-25</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>外观·组件级显示（Display Appearance 工程契约）</t>
+          <t>UI 瑕疵批修（规范 v1 待并轨清单 13 项）</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>P2</t>
+          <t>P1</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>📌 **激活 @2026-09-02（用户拍板：出工单完善验收后派活）**</t>
+          <t>裁决=MainActivity/PhotoAskSheet 文本底色取 UiTokens、primary 保 upg40 mov_prima</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>**✅ C 交付 @2026-09-01**（branch=feat/upg50，commit ca984df+8e73e8d｜A UI 编</t>
+          <t>C 完成@2026-08-29**（feat/upg25 **62986c2** 已推 origin｜含 merge origin/main</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>✅ **阶段2 复验 带缺陷通过 @2026-09-02**（ACCEPTANCE_LOG §P25：feat/upg50-ph2 5248</t>
+          <t>❌**打回@2026-08-30**：与已合 UPG-40 换肤**同文件双改**（WorkbenchPage/demo.js/MainAc</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>✅ **阶段 1 全量已合 main @2026-09-02**（0ce0fd0 链：1A f3c0fda+1B bcb18f5+1C 1a</t>
+          <t>✅**已合 main @2026-08-30**（设计师 merge 8f8debd，含 2ccce25；§六 抽查通过 13 项+候选C</t>
         </is>
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>设计师/派单/UPG-50_阶段2_MCP组件注册制开放_派单_2026-09-02.md</t>
+          <t>设计师/派单/UPG-25_重修_派单_2026-08-30.md</t>
         </is>
       </c>
       <c r="I39" t="inlineStr">
         <is>
-          <t>DEL-UPG50-20260901-001</t>
+          <t>—</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>UPG-51</t>
+          <t>UPG-26</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>用户画像标签池（Memory OS 商用投影 + 合规）</t>
+          <t>侧边栏品牌区换 logo+黑字 + 抽屉展开占比 61.8%</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
@@ -2260,22 +2260,22 @@
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>✅ 方案 v1（设计详设已补，并入 **`Memory_OS_完整设计_v2`** 附录「Commercial Projection」；定位</t>
+          <t>裁决]；用户确认已实现 @2026-09-02）→</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>**✅ C 交付 @2026-08-31**（worktree=mov-upg51 branch=feat/upg51，commit 见报告</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>审验通过 → 已合 main @2026-08-31**（设计师：ACCEPTANCE_LOG ff23a88 落档 + 查验</t>
+          <t>✅ 验收通过（用户确认「已实现」）@2026-09-02（feat/sidebar-brand 7a6dff6+0fdfe87：品牌区 lo</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>✅**验收+审验通过 → 已合 main @2026-08-31**（设计师：ACCEPTANCE_LOG ff23a88 落档 + 查验独</t>
+          <t>**分支未合 main（162 分叉）｜已合 main@2026-09-02（feat/sidebar-brand 7a6dff6/0fdf</t>
         </is>
       </c>
       <c r="H40" t="inlineStr">
@@ -2292,42 +2292,42 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>UPG-52</t>
+          <t>UPG-28</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Memory OS 生命链（Semantic 池子 + 生命周期 + Timeline + Retrieval + blockedSourceHashes）</t>
+          <t>obsidian.file.write 审批闸修复（isHarmless file.write 特判误捕）</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>P0</t>
+          <t>P1</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>✅ 方案定稿（设计依据＝`Memory_OS_完整设计_v2`，唯一口径；含验收方案）</t>
+          <t>✅**方案 v1 已出 @2026-08-29**（`设计师/方案设计/UPG-28_obsidian写入审批闸修复_方案设计.md`）</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>✅**C 完成 @2026-08-31**（认领 C worktree=mov-upg52 branch=feat/upg52，**52-1</t>
+          <t>✅**程序员 C 完成 @2026-08-30 01:05**（feat/upg28 **443b288** 已 push origin，基</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>✅**审验通过 @2026-08-31**（独立 L2 模拟器复验：memory-os 目录建立/logcat 逐字吻合/空库零影响/4 只</t>
+          <t>✅**验收员验收通过 @2026-08-30**（L1 377/0/0 亲跑+变异 M1/M2 双锚亲杀+L2 采纳模拟器证据[真机 ASK</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>✅**已合 main @2026-08-31**（设计师：§六抽查=actor 模型[AI 只 PROPOSED]/blockedSourc</t>
+          <t>✅**已合 main @443b288**（ff-only 已推 origin，合后全量复跑 377/0/0 绿；worktree mov-</t>
         </is>
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>设计师/方案设计/UPG-28_obsidian写入审批闸修复_方案设计.md</t>
         </is>
       </c>
       <c r="I41" t="inlineStr">
@@ -2339,12 +2339,12 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>UPG-53</t>
+          <t>UPG-44</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>安全体验优化改造（该守才守 · 守得舒服）</t>
+          <t>AcceptanceJudge B1 观察层（UPG-06 批2 剩项）</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
@@ -2354,27 +2354,27 @@
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>✅ 方案 v1（依据 安全体系_设计_v2.1 §5.3 + mov_安全体验_demo.html；体验优化设计+验收标准已写入文档）</t>
+          <t>裁决criteria+AI 回复→verdict/失败静默]；**投影剔键硬红**=Surface.deriveEventMessage 显</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>✅**C 完成 @2026-08-31**（feat/upg53 **a665349** 已提交 3 commit[d434ab1 8场景落</t>
+          <t>C 完成@2026-08-30 04:05**（feat/upg44 **122945b** 基底 main 3263f10 已 push；</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>✅**验收员通过+审验通过 @2026-08-31**（L1 66 套件 473/0/0 独立重跑+变异 3/3[V3/V4a/V7]+L2</t>
+          <t>审验通过 → 已合 main @2026-08-30**（设计师 §六抽查 + rebase 后 ff-only **801b8fc 已推</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>✅**已合 main @2026-08-31**（设计师：§六抽查=豁免链 gate 永不豁免写入侧已拦/vault.delete·cred</t>
+          <t>✅**验收+审验通过 → 已合 main @2026-08-30**（设计师 §六抽查 + rebase 后 ff-only **801b8</t>
         </is>
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>设计师/派单/UPG-44_AcceptanceJudge_B1_派单_2026-08-30.md</t>
         </is>
       </c>
       <c r="I42" t="inlineStr">
@@ -2386,42 +2386,42 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>UPG-54</t>
+          <t>UPG-45</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>安全中心（设置 -&gt; 安全 二级 · 等级仪表盘 + 分组策略 + 硬边界）</t>
+          <t>审批 · Approval Capability Registry（权限能力注册表）</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>P1</t>
+          <t>P0</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>✅ 方案 v2（依据 安全中心_设计_v2 + 安全体系_设计_v2.1；评审通过·有条件冻结｜等级=结果仪表盘/策略摘要/分组/审计系统级</t>
+          <t>🔨**已派单 @2026-08-30**（用户已转派；派单文本 `设计师/派单/UPG-45_审批_ApprovalRegistry_派单</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>✅**C 完成 @2026-08-31**（feat/upg54 **9911e67** 已 push origin 3 commit[47</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>✅**验收通过+审验通过 @2026-08-31**（8 项核物+482/0/0+变异 W1/W8/W5 三杀+模拟器仪表盘/实时刷新/足迹</t>
+          <t>✅**验收员通过 @2026-08-30**（ACCEPTANCE_LOG UPG-45，commit edf86d9）：核物[54行=as</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>✅**已合 main @2026-08-31**（设计师：§六抽查=SecurityCenter 等级结果仪表盘无 setGrade API</t>
+          <t>**已合 main @2026-08-31 → 审验员**（approval 体系随 UPG-58/62/63 合入；ApprovalSer</t>
         </is>
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>设计师\方案设计\审批弹窗_用户授权层_设计_v3_2026-08-30.md</t>
         </is>
       </c>
       <c r="I43" t="inlineStr">
@@ -2433,42 +2433,42 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>UPG-55</t>
+          <t>UPG-46</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>我的资产（资产管理项注册体系 · 基于安全体系 v2.1）</t>
+          <t>工具联动 Runtime 契约（Tool Orchestration）</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>P1</t>
+          <t>P0</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>✅**三轮评审采纳升 v2.2 工程冻结版 @2026-09-01**（评分 架构 9.2/安全 8.8/迁移 8.2/UI 9.1/工程</t>
+          <t>🔄 **用户拍板转交 @2026-09-05 02:19**（原认领程序员 Claude/wmw0027 做不了，用户指令转交）</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>✅**C 完成 @2026-09-01**（feat/upg55 **e1f241e** 已 push；[67-A 框架+迁移] ①Asse</t>
+          <t>✅**C 完成 @2026-09-05 03:02**（程序员 Kimi/kimi-cli，feat/upg46 **a8043aad**</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>📌 **登记丢失补录 @2026-09-02（验收员盘点发现）**：git 实证 61b2b87/27a744d/c8033b6 均已在</t>
+          <t>✅ **验收员复验通过 @2026-09-05**（§P57 落档：六件核物全在/M-cycle 锚链成立/837 差 1 双方 P3 注记</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>已合 main@2026-09-01（e1f241e）｜无遗留卡点 ｜</t>
+          <t>✅ **审验员确认+设计师合 main @7ccf0446**（2026-09-05：段①核心契约全链合入；段②=UPG-104） **卡点</t>
         </is>
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>设计师\方案设计\07_资产\我的资产_资产管理项_设计_v2_2026-08-31.md</t>
+          <t>设计师/派单/UPG-46_工具联动Runtime契约_派单_2026-09-02.md</t>
         </is>
       </c>
       <c r="I44" t="inlineStr">
@@ -2480,37 +2480,37 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>UPG-56</t>
+          <t>UPG-47</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>评测集盘点与 fixture 版本机制（改造计划第一阶段①⑤）</t>
+          <t>主页胶囊系统（pin_type+stableId / 三区 / ＋管理弹层 / 点击分派 / 长按 / 第三态 / 气泡字数）</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>P1</t>
+          <t>P0</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>✅ 方案定稿（依据 `工单方案\工单方案\改造计划+验收标准_合并版_AHE×EvoC2F_2026-08-31.md` v1.4 上篇 §</t>
+          <t>🔨已派单</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>✅**C 完成 @2026-08-31**（feat/upg56 **cc86fac** 已 push origin[1ed70a2 主体+</t>
+          <t>✅C 交付 @2026-08-30（feat/capsule-system **767228c+32ba01c** push；报告 程序员/</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>【✅ **验收员验收通过 @2026-08-31**（ACCEPTANCE_LOG c25aacf）：feat/upg56 cc86fac</t>
+          <t>✅ **验收员复验 通过 @2026-09-04**（ACCEPTANCE_LOG §P54：4e5a2f7c 隔离 worktree[申报</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>✅**审验通过+已合 main @2026-08-31**（审验 33→34：盘点报告 6 节 12 条修正口径[实测 12 条非 13]+</t>
+          <t>✅后续美化已合 main @2026-08-31（dock 对齐 **afc1ccd**：＋号圆形·随胶囊横滑·气泡左对齐胶囊；管理面板设置</t>
         </is>
       </c>
       <c r="H45" t="inlineStr">
@@ -2527,37 +2527,37 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>UPG-57</t>
+          <t>UPG-48</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Evolution Ledger 骨架（改造计划第一阶段②）</t>
+          <t>Memory API 工程契约（记忆页:memory-core/memory-api 模块化）</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>P1</t>
+          <t>P0</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>✅ 方案定稿（依据 合并版上篇 §6.1/§6.5 + 下篇 X-1/M-6；**架构约束=复用 TimelineLedger 基础设施，禁</t>
+          <t>🔨已派单 @2026-08-30</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>✅**C 完成 @2026-08-31**（feat/upg57 **f4bae35** 已 push origin[Evolution L</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>【✅ **修复复验通过 @2026-08-31**（R1｜ACCEPTANCE_LOG 04fb19f）：feat/upg57 **fbcd</t>
+          <t>❌**审验打回@2026-08-30（P1 边界违例）**｜MainActivity:582-598 直引 com.hermes.mov.m</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>✅**R1 复验通过+审验通过+已合 main @2026-08-31**（审验 33→34：NS_EVOLUTION 12 事件+ACTO</t>
+          <t>✅**已合 main @2026-08-30**（设计师 merge 92d4c22[含 0aa0c07]，审验五步复核通过：零直触core</t>
         </is>
       </c>
       <c r="H46" t="inlineStr">
@@ -2574,37 +2574,37 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>UPG-58</t>
+          <t>UPG-49</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>A-1 Manifest 五步链脚本（改造计划第一阶段③）</t>
+          <t>记忆页「我的记忆」UI 分层管理</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>P1</t>
+          <t>P2</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>✅ 方案定稿（依据 合并版上篇 A-1 + 下篇 A1-1~A1-5/M-4/M-5；**硬验=零人工步骤**，≤20 行降为推荐约束[大神</t>
+          <t>✅ 方案 v4 定稿（记忆页分层管理_设计_v4 大神 9.2 冻结）</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>✅**C 完成 @2026-08-31**（feat/upg58 **ac8d27d** 已 push origin[a62f904 主体+</t>
+          <t>🔨 **程序员 R2 修复交付 @2026-09-01**（feat/upg49-r2 **5640bce** 已 push origin</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>审验36→37：五步链+跨单消费全坐实[56 Guard 即插/57 Ledger 写入 actor=system-deriver]/L1</t>
+          <t>✅ **审验通过 @2026-09-01**（integrity_review=confirmed：P2-1a 72px 像素实证+删📌</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>✅**审验通过+已合 main @2026-08-31**（审验 36→37：五步链+跨单消费全坐实[56 Guard 即插/57 Ledg</t>
+          <t>✅ **设计师终审合流 @2026-09-02**（B9edcc4 落档+工单库补登；2 治理项裁决见下）</t>
         </is>
       </c>
       <c r="H47" t="inlineStr">
@@ -2614,66 +2614,66 @@
       </c>
       <c r="I47" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>DEL-UPG49-20260901-002</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>UPG-59</t>
+          <t>UPG-50</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>B 线蒸馏 MVP（改造计划第一阶段④ · 里程碑一承载）</t>
+          <t>外观·组件级显示（Display Appearance 工程契约）</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>P0</t>
+          <t>P2</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>✅ 方案定稿（依据 合并版上篇改造线 B + 下篇 B-1~B-9；教训六字段/三分类/配额/过期）</t>
+          <t>📌 **激活 @2026-09-02（用户拍板：出工单完善验收后派活）**</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>✅**C 完成 @2026-08-31**（feat/upg59 **8da2907** 已 push origin 2 commit[2d</t>
+          <t>**✅ C 交付 @2026-09-01**（branch=feat/upg50，commit ca984df+8e73e8d｜A UI 编</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>✅**验收通过+审验通过 @2026-08-31**（9 项核物+73 套件 519/0/0 独立重跑+变异 V4/V3b/配额三杀独立复跑</t>
+          <t>✅ **阶段2 复验 带缺陷通过 @2026-09-02**（ACCEPTANCE_LOG §P25：feat/upg50-ph2 5248</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>✅**已合 main @2026-08-31**（设计师：§六抽查=V-4 ACTIVE-only 注入过滤/配额 MAX_LESSONS=</t>
+          <t>✅ **阶段 1 全量已合 main @2026-09-02**（0ce0fd0 链：1A f3c0fda+1B bcb18f5+1C 1a</t>
         </is>
       </c>
       <c r="H48" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>设计师/派单/UPG-50_阶段2_MCP组件注册制开放_派单_2026-09-02.md</t>
         </is>
       </c>
       <c r="I48" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>DEL-UPG50-20260901-001</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>UPG-60</t>
+          <t>UPG-51</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>A-2 三道门实现+元验证（改造计划第一阶段⑥）</t>
+          <t>用户画像标签池（Memory OS 商用投影 + 合规）</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
@@ -2683,22 +2683,22 @@
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>✅ 方案定稿（依据 合并版上篇 A-2 + 下篇 A2-1~A2-6/M-1~M-6；**前置 UPG-56/58/59**）</t>
+          <t>✅ 方案 v1（设计详设已补，并入 **`Memory_OS_完整设计_v2`** 附录「Commercial Projection」；定位</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>✅**C 完成 @2026-08-31**（feat/upg60 **a8d1363** 已 push origin[5a7a576 三道门</t>
+          <t>**✅ C 交付 @2026-08-31**（worktree=mov-upg51 branch=feat/upg51，commit 见报告</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>✅**验收通过+审验通过 @2026-08-31**（9f9466d 落档：9 项测试锚+77 套件 546/0/0+变异 M1/M3v2</t>
+          <t>审验通过 → 已合 main @2026-08-31**（设计师：ACCEPTANCE_LOG ff23a88 落档 + 查验</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>✅**已合 main @2026-08-31**（设计师：§六抽查=SkillGate JS_ARTIFACT 直接拒收[A2-2 落地]/</t>
+          <t>✅**验收+审验通过 → 已合 main @2026-08-31**（设计师：ACCEPTANCE_LOG ff23a88 落档 + 查验独</t>
         </is>
       </c>
       <c r="H49" t="inlineStr">
@@ -2715,37 +2715,37 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>UPG-61</t>
+          <t>UPG-52</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>vault.get 伪放行修（记住豁免与 fail-closed handler 不一致 · UI 禁用豁免勾选）</t>
+          <t>Memory OS 生命链（Semantic 池子 + 生命周期 + Timeline + Retrieval + blockedSourceHashes）</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>P1</t>
+          <t>P0</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>定稿（UPG-53</t>
+          <t>✅ 方案定稿（设计依据＝`Memory_OS_完整设计_v2`，唯一口径；含验收方案）</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>✅**C 完成 @2026-08-31**（feat/upg61 **b7c2e9d** 已 push origin；**修法②落地·四范围</t>
+          <t>✅**C 完成 @2026-08-31**（认领 C worktree=mov-upg52 branch=feat/upg52，**52-1</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>✅ 方案定稿（UPG-53 审验员 L2 实测新发现 P1 + 设计师定夺修法；源码锚 @main 2780961：`MainActivit</t>
+          <t>✅**审验通过 @2026-08-31**（独立 L2 模拟器复验：memory-os 目录建立/logcat 逐字吻合/空库零影响/4 只</t>
         </is>
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>✅**审验通过+已合 main @2026-08-31**（审验 35→36：四范围核物+L1 74 套件 523/0/0 独立重跑+变异</t>
+          <t>✅**已合 main @2026-08-31**（设计师：§六抽查=actor 模型[AI 只 PROPOSED]/blockedSourc</t>
         </is>
       </c>
       <c r="H50" t="inlineStr">
@@ -2762,12 +2762,12 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>UPG-62</t>
+          <t>UPG-53</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>多轮对话输入框失焦修（markstream WebView 抢焦点 · 焦点归还兜底）</t>
+          <t>安全体验优化改造（该守才守 · 守得舒服）</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
@@ -2777,22 +2777,22 @@
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>✅ 方案定稿（用户真机实测报障 + 设计师溯源 @main f975437）</t>
+          <t>✅ 方案 v1（依据 安全体系_设计_v2.1 §5.3 + mov_安全体验_demo.html；体验优化设计+验收标准已写入文档）</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>✅**C 完成 @2026-08-31**（feat/upg53 **a665349** 已提交 3 commit[d434ab1 8场景落</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>✅**验收员通过+审验通过 @2026-08-31**（L1 66 套件 473/0/0 独立重跑+变异 3/3[V3/V4a/V7]+L2</t>
         </is>
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>✅**已合 main @2026-08-31**（ff-only **82c778b** 已推 origin[feat/upg61-rb 链</t>
+          <t>✅**已合 main @2026-08-31**（设计师：§六抽查=豁免链 gate 永不豁免写入侧已拦/vault.delete·cred</t>
         </is>
       </c>
       <c r="H51" t="inlineStr">
@@ -2809,12 +2809,12 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>UPG-63</t>
+          <t>UPG-54</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>第二阶段收口：弹窗基线 Z-5 + MULTI_CALL 分布统计 + M-1 真实重放补跑</t>
+          <t>安全中心（设置 -&gt; 安全 二级 · 等级仪表盘 + 分组策略 + 硬边界）</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
@@ -2824,22 +2824,22 @@
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>🔓 **五轮评审采纳升 v2.4 工程契约冻结（2026-08-31，MCP 治理评 9/10）**：67-B 范围随三细节钉死｜①审批</t>
+          <t>✅ 方案 v2（依据 安全中心_设计_v2 + 安全体系_设计_v2.1；评审通过·有条件冻结｜等级=结果仪表盘/策略摘要/分组/审计系统级</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>✅**C 完成 @2026-08-31**（feat/upg64 **115762d** 已 push origin[2d2444d 主体+</t>
+          <t>✅**C 完成 @2026-08-31**（feat/upg54 **9911e67** 已 push origin 3 commit[47</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>✅**验收+审验通过 @2026-08-31**（78 套 540/0/0+EffectSpecsTest 10/0+变异 M-64a/b</t>
+          <t>✅**验收通过+审验通过 @2026-08-31**（8 项核物+482/0/0+变异 W1/W8/W5 三杀+模拟器仪表盘/实时刷新/足迹</t>
         </is>
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>✅**已合 main @2026-08-31**（§六抽查=Registry 20 条全在+credSet/credDelete 在场[误报</t>
+          <t>✅**已合 main @2026-08-31**（设计师：§六抽查=SecurityCenter 等级结果仪表盘无 setGrade API</t>
         </is>
       </c>
       <c r="H52" t="inlineStr">
@@ -2856,12 +2856,12 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>UPG-64</t>
+          <t>UPG-55</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>C 线效应注解首批（改造计划第二阶段·C 线）</t>
+          <t>我的资产（资产管理项注册体系 · 基于安全体系 v2.1）</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
@@ -2871,27 +2871,27 @@
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>🔓 **五轮评审采纳升 v2.4 工程契约冻结（2026-08-31，MCP 治理评 9/10）**：67-B 范围随三细节钉死｜①审批</t>
+          <t>✅**三轮评审采纳升 v2.2 工程冻结版 @2026-09-01**（评分 架构 9.2/安全 8.8/迁移 8.2/UI 9.1/工程</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>✅**C 完成 @2026-08-31**（feat/upg64 **115762d** 已 push origin[2d2444d 主体+</t>
+          <t>✅**C 完成 @2026-09-01**（feat/upg55 **e1f241e** 已 push；[67-A 框架+迁移] ①Asse</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>✅**验收+审验通过 @2026-08-31**（78 套 540/0/0+EffectSpecsTest 10/0+变异 M-64a/b</t>
+          <t>📌 **登记丢失补录 @2026-09-02（验收员盘点发现）**：git 实证 61b2b87/27a744d/c8033b6 均已在</t>
         </is>
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>✅**已合 main @2026-08-31**（§六抽查=Registry 20 条全在+credSet/credDelete 在场[误报</t>
+          <t>已合 main@2026-09-01（e1f241e）｜无遗留卡点 ｜</t>
         </is>
       </c>
       <c r="H53" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>设计师\方案设计\07_资产\我的资产_资产管理项_设计_v2_2026-08-31.md</t>
         </is>
       </c>
       <c r="I53" t="inlineStr">
@@ -2903,12 +2903,12 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>UPG-65</t>
+          <t>UPG-56</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>A-2 门 3 灰度自动化（改造计划第二阶段·接 B 生产信号）</t>
+          <t>评测集盘点与 fixture 版本机制（改造计划第一阶段①⑤）</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
@@ -2918,22 +2918,22 @@
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>✅ **设计 v2 定稿 @2026-09-02**（大神二轮 12/12 全采纳｜统计口径 v2 定稿：按 skill 去重/min20+</t>
+          <t>✅ 方案定稿（依据 `工单方案\工单方案\改造计划+验收标准_合并版_AHE×EvoC2F_2026-08-31.md` v1.4 上篇 §</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>✅**C 完成 @2026-08-31**（feat/upg65 **f709ed9** 已 push origin[e4aa2a6 主体+</t>
+          <t>✅**C 完成 @2026-08-31**（feat/upg56 **cc86fac** 已 push origin[1ed70a2 主体+</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>⚠️ **错挂注记 @2026-09-05（设计师）**：以下打回段主体=feat/upg63 0580fa8，属 **UPG-63** 卡</t>
+          <t>【✅ **验收员验收通过 @2026-08-31**（ACCEPTANCE_LOG c25aacf）：feat/upg56 cc86fac</t>
         </is>
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>✅ **已合 main @34c37f54（补登 @2026-09-05，设计师核物）**：=交付提交 e4aa2a6 的 patch-id</t>
+          <t>✅**审验通过+已合 main @2026-08-31**（审验 33→34：盘点报告 6 节 12 条修正口径[实测 12 条非 13]+</t>
         </is>
       </c>
       <c r="H54" t="inlineStr">
@@ -2950,37 +2950,37 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>UPG-66</t>
+          <t>UPG-57</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>A-3 Judge 扩面（改造计划第二阶段·判定三类+反哺管道）</t>
+          <t>Evolution Ledger 骨架（改造计划第一阶段②）</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>P2</t>
+          <t>P1</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>✅ 方案定稿（依据 合并版上篇 A-3 + 下篇 A3-1~A3-4；独立可随时插队）</t>
+          <t>✅ 方案定稿（依据 合并版上篇 §6.1/§6.5 + 下篇 X-1/M-6；**架构约束=复用 TimelineLedger 基础设施，禁</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>✅**C 完成 @2026-08-31**（feat/upg66 **1e604c7** 已 push origin[0438049 主体+</t>
+          <t>✅**C 完成 @2026-08-31**（feat/upg57 **f4bae35** 已 push origin[Evolution L</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>【✅ **验收员验收通过 @2026-08-31**（ACCEPTANCE_LOG 9e764fb）：feat/upg66 1e604c7</t>
+          <t>【✅ **修复复验通过 @2026-08-31**（R1｜ACCEPTANCE_LOG 04fb19f）：feat/upg57 **fbcd</t>
         </is>
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t>✅ **已合 main@2026-09-01**（A-3 Judge 扩面｜AcceptanceJudge/M-JudgeModes/Age</t>
+          <t>✅**R1 复验通过+审验通过+已合 main @2026-08-31**（审验 33→34：NS_EVOLUTION 12 事件+ACTO</t>
         </is>
       </c>
       <c r="H55" t="inlineStr">
@@ -2997,37 +2997,37 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>UPG-67</t>
+          <t>UPG-58</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>D 线 DAG 编排试点（改造计划第三阶段 · 预立待前置）</t>
+          <t>A-1 Manifest 五步链脚本（改造计划第一阶段③）</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>P2</t>
+          <t>P1</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>✅ 方案定稿（依据 合并版上篇改造线 D + 下篇 D-1~D-5 + §十三 执行细则）</t>
+          <t>✅ 方案定稿（依据 合并版上篇 A-1 + 下篇 A1-1~A1-5/M-4/M-5；**硬验=零人工步骤**，≤20 行降为推荐约束[大神</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>✅**C 完成 @2026-08-31**（feat/upg67 **040c9d9** 已 push origin[a88510a 主体+</t>
+          <t>✅**C 完成 @2026-08-31**（feat/upg58 **ac8d27d** 已 push origin[a62f904 主体+</t>
         </is>
       </c>
       <c r="F56" t="inlineStr">
         <is>
-          <t>【✅ **验收员验收通过 @2026-09-01**（ACCEPTANCE_LOG 6f330b5）：feat/upg67 040c9d9；</t>
+          <t>审验36→37：五步链+跨单消费全坐实[56 Guard 即插/57 Ledger 写入 actor=system-deriver]/L1</t>
         </is>
       </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t>✅**已合 main @2026-08-31**（§六抽查=DagPlanner cycle 拒绝[Kahn 失败→Reject 不 han</t>
+          <t>✅**审验通过+已合 main @2026-08-31**（审验 36→37：五步链+跨单消费全坐实[56 Guard 即插/57 Ledg</t>
         </is>
       </c>
       <c r="H56" t="inlineStr">
@@ -3044,12 +3044,12 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>UPG-68</t>
+          <t>UPG-59</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>商业安全闸（原「商业防线批」——W2 白名单自动闸 + 商业面 fail-open 集中收口）</t>
+          <t>B 线蒸馏 MVP（改造计划第一阶段④ · 里程碑一承载）</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
@@ -3059,27 +3059,27 @@
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>✅ **设计 v1 定稿 @2026-09-01**（`设计师\方案设计\05_审批\审批白名单机器可读化与注册即校验_设计_v1_2026</t>
+          <t>✅ 方案定稿（依据 合并版上篇改造线 B + 下篇 B-1~B-9；教训六字段/三分类/配额/过期）</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>✅ **C 完成 @2026-09-02**（补充节 V68-8/V69-4 补验：feat/upg68 `8380108`；变异亲杀 4/</t>
+          <t>✅**C 完成 @2026-08-31**（feat/upg59 **8da2907** 已 push origin 2 commit[2d</t>
         </is>
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t>✅ R1 复验带缺陷通过 @2026-09-01（feat/upg68 35b0008｜HIGH/M1/M2 三缺口 security_re</t>
+          <t>✅**验收通过+审验通过 @2026-08-31**（9 项核物+73 套件 519/0/0 独立重跑+变异 V4/V3b/配额三杀独立复跑</t>
         </is>
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>✅ **已合 main @c2defad @2026-09-02**（rebase origin/main 零冲突 + ff；V68-8/V</t>
+          <t>✅**已合 main @2026-08-31**（设计师：§六抽查=V-4 ACTIVE-only 注入过滤/配额 MAX_LESSONS=</t>
         </is>
       </c>
       <c r="H57" t="inlineStr">
         <is>
-          <t>设计师\方案设计\05_审批\审批白名单机器可读化与注册即校验_设计_v1_2026-09-01.md</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I57" t="inlineStr">
@@ -3091,12 +3091,12 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>UPG-69</t>
+          <t>UPG-60</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>WebMCP 站点试点（mow.kim 工单站「站点=业务工具」第一站）</t>
+          <t>A-2 三道门实现+元验证（改造计划第一阶段⑥）</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
@@ -3106,22 +3106,22 @@
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>已派单（用户直接外派 @2026-09-05——撤销改向挂起，原 mow.kim 工单站口径继续）</t>
+          <t>✅ 方案定稿（依据 合并版上篇 A-2 + 下篇 A2-1~A2-6/M-1~M-6；**前置 UPG-56/58/59**）</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>✅**C 完成 @2026-08-31**（feat/upg60 **a8d1363** 已 push origin[5a7a576 三道门</t>
         </is>
       </c>
       <c r="F58" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>✅**验收通过+审验通过 @2026-08-31**（9f9466d 落档：9 项测试锚+77 套件 546/0/0+变异 M1/M3v2</t>
         </is>
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>改向挂起：试点职能由 UPG-105 批二承接，工单三工具留商家后台线</t>
+          <t>✅**已合 main @2026-08-31**（设计师：§六抽查=SkillGate JS_ARTIFACT 直接拒收[A2-2 落地]/</t>
         </is>
       </c>
       <c r="H58" t="inlineStr">
@@ -3138,15 +3138,438 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
+          <t>UPG-61</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>vault.get 伪放行修（记住豁免与 fail-closed handler 不一致 · UI 禁用豁免勾选）</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>定稿（UPG-53</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>✅**C 完成 @2026-08-31**（feat/upg61 **b7c2e9d** 已 push origin；**修法②落地·四范围</t>
+        </is>
+      </c>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>✅ 方案定稿（UPG-53 审验员 L2 实测新发现 P1 + 设计师定夺修法；源码锚 @main 2780961：`MainActivit</t>
+        </is>
+      </c>
+      <c r="G59" t="inlineStr">
+        <is>
+          <t>✅**审验通过+已合 main @2026-08-31**（审验 35→36：四范围核物+L1 74 套件 523/0/0 独立重跑+变异</t>
+        </is>
+      </c>
+      <c r="H59" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I59" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>UPG-62</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>多轮对话输入框失焦修（markstream WebView 抢焦点 · 焦点归还兜底）</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>✅ 方案定稿（用户真机实测报障 + 设计师溯源 @main f975437）</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G60" t="inlineStr">
+        <is>
+          <t>✅**已合 main @2026-08-31**（ff-only **82c778b** 已推 origin[feat/upg61-rb 链</t>
+        </is>
+      </c>
+      <c r="H60" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I60" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>UPG-63</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>第二阶段收口：弹窗基线 Z-5 + MULTI_CALL 分布统计 + M-1 真实重放补跑</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>🔓 **五轮评审采纳升 v2.4 工程契约冻结（2026-08-31，MCP 治理评 9/10）**：67-B 范围随三细节钉死｜①审批</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>✅**C 完成 @2026-08-31**（feat/upg64 **115762d** 已 push origin[2d2444d 主体+</t>
+        </is>
+      </c>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>✅**验收+审验通过 @2026-08-31**（78 套 540/0/0+EffectSpecsTest 10/0+变异 M-64a/b</t>
+        </is>
+      </c>
+      <c r="G61" t="inlineStr">
+        <is>
+          <t>✅**已合 main @2026-08-31**（§六抽查=Registry 20 条全在+credSet/credDelete 在场[误报</t>
+        </is>
+      </c>
+      <c r="H61" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I61" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>UPG-64</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>C 线效应注解首批（改造计划第二阶段·C 线）</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>🔓 **五轮评审采纳升 v2.4 工程契约冻结（2026-08-31，MCP 治理评 9/10）**：67-B 范围随三细节钉死｜①审批</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>✅**C 完成 @2026-08-31**（feat/upg64 **115762d** 已 push origin[2d2444d 主体+</t>
+        </is>
+      </c>
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>✅**验收+审验通过 @2026-08-31**（78 套 540/0/0+EffectSpecsTest 10/0+变异 M-64a/b</t>
+        </is>
+      </c>
+      <c r="G62" t="inlineStr">
+        <is>
+          <t>✅**已合 main @2026-08-31**（§六抽查=Registry 20 条全在+credSet/credDelete 在场[误报</t>
+        </is>
+      </c>
+      <c r="H62" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I62" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>UPG-65</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>A-2 门 3 灰度自动化（改造计划第二阶段·接 B 生产信号）</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>✅ **设计 v2 定稿 @2026-09-02**（大神二轮 12/12 全采纳｜统计口径 v2 定稿：按 skill 去重/min20+</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>✅**C 完成 @2026-08-31**（feat/upg65 **f709ed9** 已 push origin[e4aa2a6 主体+</t>
+        </is>
+      </c>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>⚠️ **错挂注记 @2026-09-05（设计师）**：以下打回段主体=feat/upg63 0580fa8，属 **UPG-63** 卡</t>
+        </is>
+      </c>
+      <c r="G63" t="inlineStr">
+        <is>
+          <t>✅ **已合 main @34c37f54（补登 @2026-09-05，设计师核物）**：=交付提交 e4aa2a6 的 patch-id</t>
+        </is>
+      </c>
+      <c r="H63" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I63" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>UPG-66</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>A-3 Judge 扩面（改造计划第二阶段·判定三类+反哺管道）</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>✅ 方案定稿（依据 合并版上篇 A-3 + 下篇 A3-1~A3-4；独立可随时插队）</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>✅**C 完成 @2026-08-31**（feat/upg66 **1e604c7** 已 push origin[0438049 主体+</t>
+        </is>
+      </c>
+      <c r="F64" t="inlineStr">
+        <is>
+          <t>【✅ **验收员验收通过 @2026-08-31**（ACCEPTANCE_LOG 9e764fb）：feat/upg66 1e604c7</t>
+        </is>
+      </c>
+      <c r="G64" t="inlineStr">
+        <is>
+          <t>✅ **已合 main@2026-09-01**（A-3 Judge 扩面｜AcceptanceJudge/M-JudgeModes/Age</t>
+        </is>
+      </c>
+      <c r="H64" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I64" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>UPG-67</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>D 线 DAG 编排试点（改造计划第三阶段 · 预立待前置）</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>✅ 方案定稿（依据 合并版上篇改造线 D + 下篇 D-1~D-5 + §十三 执行细则）</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>✅**C 完成 @2026-08-31**（feat/upg67 **040c9d9** 已 push origin[a88510a 主体+</t>
+        </is>
+      </c>
+      <c r="F65" t="inlineStr">
+        <is>
+          <t>【✅ **验收员验收通过 @2026-09-01**（ACCEPTANCE_LOG 6f330b5）：feat/upg67 040c9d9；</t>
+        </is>
+      </c>
+      <c r="G65" t="inlineStr">
+        <is>
+          <t>✅**已合 main @2026-08-31**（§六抽查=DagPlanner cycle 拒绝[Kahn 失败→Reject 不 han</t>
+        </is>
+      </c>
+      <c r="H65" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I65" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>UPG-68</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>商业安全闸（原「商业防线批」——W2 白名单自动闸 + 商业面 fail-open 集中收口）</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>✅ **设计 v1 定稿 @2026-09-01**（`设计师\方案设计\05_审批\审批白名单机器可读化与注册即校验_设计_v1_2026</t>
+        </is>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>✅ **C 完成 @2026-09-02**（补充节 V68-8/V69-4 补验：feat/upg68 `8380108`；变异亲杀 4/</t>
+        </is>
+      </c>
+      <c r="F66" t="inlineStr">
+        <is>
+          <t>✅ R1 复验带缺陷通过 @2026-09-01（feat/upg68 35b0008｜HIGH/M1/M2 三缺口 security_re</t>
+        </is>
+      </c>
+      <c r="G66" t="inlineStr">
+        <is>
+          <t>✅ **已合 main @c2defad @2026-09-02**（rebase origin/main 零冲突 + ff；V68-8/V</t>
+        </is>
+      </c>
+      <c r="H66" t="inlineStr">
+        <is>
+          <t>设计师\方案设计\05_审批\审批白名单机器可读化与注册即校验_设计_v1_2026-09-01.md</t>
+        </is>
+      </c>
+      <c r="I66" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>UPG-69</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>WebMCP 站点试点（mow.kim 工单站「站点=业务工具」第一站）</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>📌 已派单（用户直接外派）</t>
+        </is>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>✅ C 完成 @2026-09-05（f5e7212a——站点三件+3 端点+契约锚；DEL 挂起已随 STD 补冻解锁；待验收）</t>
+        </is>
+      </c>
+      <c r="F67" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G67" t="inlineStr">
+        <is>
+          <t>改向挂起：试点职能由 UPG-105 批二承接，工单三工具留商家后台线</t>
+        </is>
+      </c>
+      <c r="H67" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I67" t="inlineStr">
+        <is>
+          <t>DEL-UPG69-20260905-001</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
           <t>UPG-70</t>
         </is>
       </c>
-      <c r="B59" t="inlineStr">
+      <c r="B68" t="inlineStr">
         <is>
           <t>UI 组件化改造 · 地基（单一数据源/形态类归层/规范对齐）</t>
         </is>
       </c>
-      <c r="C59" t="inlineStr">
+      <c r="C68" t="inlineStr">
         <is>
           <t>P2
 → **审验**：✅ 通过 @2026-09-02（integrity_review=confirmed，与 ACCEPTANCE_LOG §P26 一致——合入版 667cc80 与 b47ecb8 patch-id 等价逐字节一致；基线 2 失败亲跑对照坐实=收拢版带病预存、UPG-70 零新增失败；A1/A2 核物全坐实）；3 条 P3 不阻塞（①交付报告落点已移 程序员\交付报告\ ②manifest 缺口→挂账 ③autocrlf 误报→CI 权威）
@@ -3156,190 +3579,190 @@
 → **依据**：2026-09-02 调研 GitHub 成熟方案</t>
         </is>
       </c>
-      <c r="D59" t="inlineStr">
+      <c r="D68" t="inlineStr">
         <is>
           <t>**裁决**（用户拍板 2026-09-02）：基线 2 失败=**契约锚同步修**（AppearanceContractTest 适配收拢</t>
         </is>
       </c>
-      <c r="E59" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F59" t="inlineStr">
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F68" t="inlineStr">
         <is>
           <t>**验收**：验收员复验 带缺陷通过 @2026-09-02（ACCEPTANCE_LOG §P26：b47ecb8 隔离 worktree</t>
         </is>
       </c>
-      <c r="G59" t="inlineStr">
+      <c r="G68" t="inlineStr">
         <is>
           <t>✅ 已合 main @667cc80（feat/upg70 b47ecb8 cherry-pick 667cc80）｜ DONE</t>
         </is>
       </c>
-      <c r="H59" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I59" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-    </row>
-    <row r="60">
-      <c r="A60" t="inlineStr">
+      <c r="H68" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I68" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
         <is>
           <t>UPG-71</t>
         </is>
       </c>
-      <c r="B60" t="inlineStr">
+      <c r="B69" t="inlineStr">
         <is>
           <t>元能力注册表 · 地基（MVP 资产 + Schema + 校验脚本）</t>
         </is>
       </c>
-      <c r="C60" t="inlineStr">
+      <c r="C69" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
-      <c r="D60" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E60" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F60" t="inlineStr">
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F69" t="inlineStr">
         <is>
           <t>✅ **审验 通过 @2026-09-02**（integrity_review 与 §P27 一致｜L1①/②/④/⑤ 亲跑全坐实；观察</t>
         </is>
       </c>
-      <c r="G60" t="inlineStr">
+      <c r="G69" t="inlineStr">
         <is>
           <t>✅ 已合 main @43fd00a（feat/upg71 快进合入+已 push）｜ DONE</t>
         </is>
       </c>
-      <c r="H60" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I60" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-    </row>
-    <row r="61">
-      <c r="A61" t="inlineStr">
+      <c r="H69" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I69" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
         <is>
           <t>UPG-72</t>
         </is>
       </c>
-      <c r="B61" t="inlineStr">
+      <c r="B70" t="inlineStr">
         <is>
           <t>执行引擎 · S2 JobSpec+SchemaGate+READ 直跑（契约 v0.4 首接线单）</t>
         </is>
       </c>
-      <c r="C61" t="inlineStr">
+      <c r="C70" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
-      <c r="D61" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E61" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F61" t="inlineStr">
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F70" t="inlineStr">
         <is>
           <t>✅ **审验 通过 @2026-09-02**（§P28 一致：红线边界 diff 17 文件全模块零触碰、mov-exec-engine:</t>
         </is>
       </c>
-      <c r="G61" t="inlineStr">
+      <c r="G70" t="inlineStr">
         <is>
           <t>✅ **设计师合 main**：bd958d2（父=main 43fd00a，快进） **前置**：✅ UPG-71 已合 main @43</t>
         </is>
       </c>
-      <c r="H61" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I61" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-    </row>
-    <row r="62">
-      <c r="A62" t="inlineStr">
+      <c r="H70" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I70" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
         <is>
           <t>UPG-73</t>
         </is>
       </c>
-      <c r="B62" t="inlineStr">
+      <c r="B71" t="inlineStr">
         <is>
           <t>执行引擎 · S3 审批双快照核心（ApprovalSnapshot+首决胜+STALE）+ WRITE/MONEY 接审批（契约 v0.4 第二条接线单）</t>
         </is>
       </c>
-      <c r="C62" t="inlineStr">
+      <c r="C71" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
-      <c r="D62" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E62" t="inlineStr">
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E71" t="inlineStr">
         <is>
           <t>✅ **R1 修复交付 @2026-09-02**（程序员 feat/upg73 **add9e8c**：HIGH ApprovalBook</t>
         </is>
       </c>
-      <c r="F62" t="inlineStr">
+      <c r="F71" t="inlineStr">
         <is>
           <t>✅ **审验 通过 @2026-09-02**（§P29-R1 consistent：R1 范围 5 文件+273/-31 限 approv</t>
         </is>
       </c>
-      <c r="G62" t="inlineStr">
+      <c r="G71" t="inlineStr">
         <is>
           <t>✅ **已合 main @add9e8c**（快进合入+已 push；元能力线合序 71→72→73 完成）｜ DONE **前置**：✅</t>
         </is>
       </c>
-      <c r="H62" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I62" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-    </row>
-    <row r="63">
-      <c r="A63" t="inlineStr">
+      <c r="H71" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I71" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
         <is>
           <t>UPG-75</t>
         </is>
       </c>
-      <c r="B63" t="inlineStr">
+      <c r="B72" t="inlineStr">
         <is>
           <t>审批交互收口（弹窗队列/待办列表/渠道统一）</t>
         </is>
       </c>
-      <c r="C63" t="inlineStr">
+      <c r="C72" t="inlineStr">
         <is>
           <t>P1
 → **验收链**：验收员复验 带缺陷通过（§P30：A1 首决胜真 CAS[ApprovalService:196-200 AtomicReference + compareAndSet 非 check-then-act——UPG-73 教训内化]+FIFO 队列+待办 chip/面板+单源收口；A3-1 渠道端到端 JVM 无法覆盖[远程面触发不达 UI——模拟器环境阻塞]）→ ✅ 审验通过（014c10f 4 文件+650/-109 纯交互层；A1-1 变异亲杀[keep-latest→A1-1 红→还原复绿]；红线边界[only-once/fail-closed 零改动]）
@@ -3347,191 +3770,191 @@
 → **依据**：审批安全语义</t>
         </is>
       </c>
-      <c r="D63" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E63" t="inlineStr">
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E72" t="inlineStr">
         <is>
           <t>✅ **C 交付 @2026-09-02**（程序员 feat/upg75 **014c10f**，worktree mov-upg75，基</t>
         </is>
       </c>
-      <c r="F63" t="inlineStr">
+      <c r="F72" t="inlineStr">
         <is>
           <t>✅ **验收员复验 带缺陷通过 @2026-09-02**（ACCEPTANCE_LOG §P30：014c10f 隔离 worktree｜</t>
         </is>
       </c>
-      <c r="G63" t="inlineStr">
+      <c r="G72" t="inlineStr">
         <is>
           <t>✅ 已合 main @014c10f（feat/upg75 ff 合入；本地合入完成｜push 待网络恢复）｜ DONE（待 push）</t>
         </is>
       </c>
-      <c r="H63" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I63" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-    </row>
-    <row r="64">
-      <c r="A64" t="inlineStr">
+      <c r="H72" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I72" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
         <is>
           <t>UPG-76</t>
         </is>
       </c>
-      <c r="B64" t="inlineStr">
+      <c r="B73" t="inlineStr">
         <is>
           <t>审批预审单模式（先扫一遍→审批单→同意就做）</t>
         </is>
       </c>
-      <c r="C64" t="inlineStr">
+      <c r="C73" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
-      <c r="D64" t="inlineStr">
+      <c r="D73" t="inlineStr">
         <is>
           <t>📎 **方案 v2 增补 @2026-09-03**（设计师B「四钉子」，用户已认可：`设计师\方案设计\审批预审单_UPG-76_方案v</t>
         </is>
       </c>
-      <c r="E64" t="inlineStr">
+      <c r="E73" t="inlineStr">
         <is>
           <t>✅ **C 交付 @2026-09-03**（程序员 feat/upg76 **ed5088c**，worktree mov-upg76，基</t>
         </is>
       </c>
-      <c r="F64" t="inlineStr">
+      <c r="F73" t="inlineStr">
         <is>
           <t>✅ **验收员复验 带缺陷通过 @2026-09-03**（ACCEPTANCE_LOG §P32：ed5088c 隔离 worktree｜</t>
         </is>
       </c>
-      <c r="G64" t="inlineStr">
+      <c r="G73" t="inlineStr">
         <is>
           <t>✅ **已合 main @6dd9161 @2026-09-03**（设计师B：ff-only 合入+**已 push origin/mai</t>
         </is>
       </c>
-      <c r="H64" t="inlineStr">
+      <c r="H73" t="inlineStr">
         <is>
           <t>设计师\派单\UPG-76_审批预审单_派单_2026-09-03.md</t>
         </is>
       </c>
-      <c r="I64" t="inlineStr">
+      <c r="I73" t="inlineStr">
         <is>
           <t>DEL-UPG76-20260903-001</t>
         </is>
       </c>
     </row>
-    <row r="65">
-      <c r="A65" t="inlineStr">
+    <row r="74">
+      <c r="A74" t="inlineStr">
         <is>
           <t>UPG-77</t>
         </is>
       </c>
-      <c r="B65" t="inlineStr">
+      <c r="B74" t="inlineStr">
         <is>
           <t>审批判定单源化 + MCP 面死信通道处置 + SDK 契约纠偏（P0 安全）</t>
         </is>
       </c>
-      <c r="C65" t="inlineStr">
+      <c r="C74" t="inlineStr">
         <is>
           <t>P0</t>
         </is>
       </c>
-      <c r="D65" t="inlineStr">
+      <c r="D74" t="inlineStr">
         <is>
           <t>📌 已派单·待认领（派单 `设计师\派单\UPG-77_审批判定单源化_派单_2026-09-03.md`；验收标准已冻结 `STD-UP</t>
         </is>
       </c>
-      <c r="E65" t="inlineStr">
+      <c r="E74" t="inlineStr">
         <is>
           <t>✅ **C 交付 @2026-09-03**（程序员 feat/upg77 **a7736b3**，worktree mov-upg77，基</t>
         </is>
       </c>
-      <c r="F65" t="inlineStr">
+      <c r="F74" t="inlineStr">
         <is>
           <t>✅ **验收员复验 通过 @2026-09-03**（ACCEPTANCE_LOG §P31：a7736b3 隔离 worktree｜全量</t>
         </is>
       </c>
-      <c r="G65" t="inlineStr">
+      <c r="G74" t="inlineStr">
         <is>
           <t>✅ **已合 main @a7736b3 @2026-09-03**（设计师B：ff-only 合入 + **已 push origin/m</t>
         </is>
       </c>
-      <c r="H65" t="inlineStr">
+      <c r="H74" t="inlineStr">
         <is>
           <t>设计师\派单\UPG-77_审批判定单源化_派单_2026-09-03.md</t>
         </is>
       </c>
-      <c r="I65" t="inlineStr">
+      <c r="I74" t="inlineStr">
         <is>
           <t>DEL-UPG77-20260903-001</t>
         </is>
       </c>
     </row>
-    <row r="66">
-      <c r="A66" t="inlineStr">
+    <row r="75">
+      <c r="A75" t="inlineStr">
         <is>
           <t>UPG-78</t>
         </is>
       </c>
-      <c r="B66" t="inlineStr">
+      <c r="B75" t="inlineStr">
         <is>
           <t>生成器派生项入库保鲜 + CI diff=0 门禁（ApprovalRegistry 系）</t>
         </is>
       </c>
-      <c r="C66" t="inlineStr">
+      <c r="C75" t="inlineStr">
         <is>
           <t>P2 → ✅ **验收员复验 通过 @2026-09-03**（ACCEPTANCE_LOG §P33：f1e2067 隔离 worktree 三锚行为级复现——A1 删 inventory→dependsOn 自动重建+722/2/1[GeneratorTest 不再红=**§P25 P2-A2 闭环**]+A3 连跑两遍 md5 一致+内容零 drift[status M=CRLF 假差异]+A2 CI git diff --exit-code 门禁；manifest_sha 一致 ok:True；**§P25/§P27/§P30 三处生成器漂移遗留根治闭环**；**达待合→设计师**[CI 首跑回看=A2 终证]）
 → ✅ **已合 main @f1e2067 @2026-09-03**</t>
         </is>
       </c>
-      <c r="D66" t="inlineStr">
+      <c r="D75" t="inlineStr">
         <is>
           <t>📌 **已派单·待认领 @2026-09-03**（用户拍板「一起干了」；派单 `设计师\派单\UPG-78_生成器门禁_派单_2026-</t>
         </is>
       </c>
-      <c r="E66" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F66" t="inlineStr">
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F75" t="inlineStr">
         <is>
           <t>✅ **验收员复验 通过 @2026-09-03**（ACCEPTANCE_LOG §P33：f1e2067 隔离 worktree 三锚行</t>
         </is>
       </c>
-      <c r="G66" t="inlineStr">
+      <c r="G75" t="inlineStr">
         <is>
           <t>✅ **已合 main @f1e2067 @2026-09-03**（设计师B：ff-only 合入+**已 push origin/mai</t>
         </is>
       </c>
-      <c r="H66" t="inlineStr">
+      <c r="H75" t="inlineStr">
         <is>
           <t>设计师\派单\UPG-78_生成器门禁_派单_2026-09-03.md</t>
         </is>
       </c>
-      <c r="I66" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-    </row>
-    <row r="67">
-      <c r="A67" t="inlineStr">
+      <c r="I75" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
         <is>
           <t>UPG-79</t>
         </is>
       </c>
-      <c r="B67" t="inlineStr">
+      <c r="B76" t="inlineStr">
         <is>
           <t>审批呈现层组件化（ApprovalSurface + CardShell v1 视觉 + 渠道三修）</t>
         </is>
       </c>
-      <c r="C67" t="inlineStr">
+      <c r="C76" t="inlineStr">
         <is>
           <t>P1 → ✅ **验收员复验 带缺陷通过 @2026-09-03**（ACCEPTANCE_LOG §P34：3925561 隔离 worktree——全量 734/2/1 亲跑一致+ApprovalLogic 9 用例+**变异④ 亲杀**[only-once 勾选禁则]+红线零改动；L2 CARD v2 采信程序员 4 图实证[同 AVD+呈现机制 UPG-77 已实证]+验收员抽验受阻如实记录；受限 3 项真机复验专项待环境恢复；**达待合→审验员→设计师**）
 → ✅ **已合 main @5cf546d @2026-09-03**（设计师B：rebase f1e2067 后 ff-only 合入+**已 push origin/main**——rebase 前后 patch-id 4d645861 逐字节等价实证[3925561≡5cf546d]，合后定向 ApprovalLogic/ComponentContract/ApprovalQueue BUILD SUCCESSFUL；合前抽查[红线 15/§六]——STD-UPG-79-v1 sha=97f756ff 对账一致、§P34 证据=代码核物+变异亲杀实物；**用户视觉反馈处置**：截图灰带（#ECECEC）经网格采样+colors.xml+最终代码三方核对=**3925561 已无此灰带**（卡体纯白、勾选行无背景，与用户要求一致，截图疑为 WIP 版）——若新包仍见灰带按 P3 新单追）
@@ -3539,49 +3962,49 @@
 → **依据**：总纲 v1「L2 呈现层=体系唯一黑洞」+ 评审增补——UPG-75 呈现为散装内联实现</t>
         </is>
       </c>
-      <c r="D67" t="inlineStr">
+      <c r="D76" t="inlineStr">
         <is>
           <t>📌 **已派单·待认领 @2026-09-03**（总纲 R1=审批体系最后一块，用户拍板派出；派单 `设计师\派单\UPG-79_审批呈</t>
         </is>
       </c>
-      <c r="E67" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F67" t="inlineStr">
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F76" t="inlineStr">
         <is>
           <t>✅ **验收员复验 带缺陷通过 @2026-09-03**（ACCEPTANCE_LOG §P34：3925561 隔离 worktree｜</t>
         </is>
       </c>
-      <c r="G67" t="inlineStr">
+      <c r="G76" t="inlineStr">
         <is>
           <t>✅ **已合 main @5cf546d @2026-09-03**（设计师B：rebase f1e2067 后 ff-only 合入+**</t>
         </is>
       </c>
-      <c r="H67" t="inlineStr">
+      <c r="H76" t="inlineStr">
         <is>
           <t>设计师\派单\UPG-79_审批呈现层组件化_派单_2026-09-03.md</t>
         </is>
       </c>
-      <c r="I67" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-    </row>
-    <row r="68">
-      <c r="A68" t="inlineStr">
+      <c r="I76" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
         <is>
           <t>UPG-80</t>
         </is>
       </c>
-      <c r="B68" t="inlineStr">
+      <c r="B77" t="inlineStr">
         <is>
           <t>AI 对话链路诊断修复（模拟器 DeepSeek 链路）+ 联动补验</t>
         </is>
       </c>
-      <c r="C68" t="inlineStr">
+      <c r="C77" t="inlineStr">
         <is>
           <t>P1（验证环境根） → ✅ **验收员复验 通过 @2026-09-03**（ACCEPTANCE_LOG §P36：零代码诊断单复核通过——A1 诊断证据在档[AI 未回复挂账可销]；**A3 UPG-76 场景① 全链实证补入**[预审单四段全实证——§P32 场景① 阻塞解除]；场景③④✅+② ⛔ payment mock 待接；**removeAll 缺陷实锤转单**[批量写同工具名被砍单——MainActivity:5543]）
 → ✅ **已闭环 @2026-09-03**（零代码单无合 main 对象：验收员 §P36 + 审验 confirmed——A1 诊断 logcat 全链路健康在档[首查截断误判取全文核实]、联动 UPG-76 L3 ①③④ 全实证[预审单六锚/已批执行+未批阻断+计划外新窗/门槛单步弹窗]、脱敏闸 54 文件零非打码 key；挂账-模拟器AI未回复 已销、挂账-upg76-L3 ①③④ 已实证仅剩② MONEY 转 挂账-payment.pay handler缺失；审验发现① removeAll 缺陷已转 UPG-85 P1）
@@ -3590,191 +4013,191 @@
 → ✅ **C 交付 @2026-09-03**</t>
         </is>
       </c>
-      <c r="D68" t="inlineStr">
+      <c r="D77" t="inlineStr">
         <is>
           <t>📌 **已派单·待认领 @2026-09-03**（派单 `设计师\派单\UPG-80_AI对话链路修复_派单_2026-09-03.md</t>
         </is>
       </c>
-      <c r="E68" t="inlineStr">
+      <c r="E77" t="inlineStr">
         <is>
           <t>✅ **C 交付 @2026-09-03**（程序员 Claude/wmw0027，**零代码改动**｜A2 判定纯环境/配置面，无代码缺陷</t>
         </is>
       </c>
-      <c r="F68" t="inlineStr">
+      <c r="F77" t="inlineStr">
         <is>
           <t>✅ **验收员复验 通过 @2026-09-03**（ACCEPTANCE_LOG §P36：零代码诊断单复核通过｜A1 诊断证据在档[AI</t>
         </is>
       </c>
-      <c r="G68" t="inlineStr">
+      <c r="G77" t="inlineStr">
         <is>
           <t>✅ **已闭环 @2026-09-03**（零代码单无合 main 对象：验收员 §P36 + 审验 confirmed｜A1 诊断 log</t>
         </is>
       </c>
-      <c r="H68" t="inlineStr">
+      <c r="H77" t="inlineStr">
         <is>
           <t>设计师\派单\UPG-80_AI对话链路修复_派单_2026-09-03.md</t>
         </is>
       </c>
-      <c r="I68" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-    </row>
-    <row r="69">
-      <c r="A69" t="inlineStr">
+      <c r="I77" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
         <is>
           <t>UPG-81</t>
         </is>
       </c>
-      <c r="B69" t="inlineStr">
+      <c r="B78" t="inlineStr">
         <is>
           <t>基线 2 失败契约锚同步修（AppearanceContractTest 适配收拢版现实）</t>
         </is>
       </c>
-      <c r="C69" t="inlineStr">
+      <c r="C78" t="inlineStr">
         <is>
           <t>P2</t>
         </is>
       </c>
-      <c r="D69" t="inlineStr">
+      <c r="D78" t="inlineStr">
         <is>
           <t>📌 **已派单·待认领 @2026-09-03**（派单 `设计师\派单\UPG-81_基线契约锚同步修_派单_2026-09-03.md</t>
         </is>
       </c>
-      <c r="E69" t="inlineStr">
+      <c r="E78" t="inlineStr">
         <is>
           <t>✅ **C 交付 @2026-09-03 09:19**（程序员 Claude/wmw0027，commit 3339c4b @feat/u</t>
         </is>
       </c>
-      <c r="F69" t="inlineStr">
+      <c r="F78" t="inlineStr">
         <is>
           <t>✅ **验收员复验 通过 @2026-09-03**（ACCEPTANCE_LOG §P39：8609d69 隔离 worktree</t>
         </is>
       </c>
-      <c r="G69" t="inlineStr">
+      <c r="G78" t="inlineStr">
         <is>
           <t>✅ **已合 main（补登 @2026-09-05）**（审验员 09-05 核实：3339c4b patch-id≡**fab7d29*</t>
         </is>
       </c>
-      <c r="H69" t="inlineStr">
+      <c r="H78" t="inlineStr">
         <is>
           <t>设计师\派单\UPG-81_基线契约锚同步修_派单_2026-09-03.md</t>
         </is>
       </c>
-      <c r="I69" t="inlineStr">
+      <c r="I78" t="inlineStr">
         <is>
           <t>DEL-UPG81-20260903-001</t>
         </is>
       </c>
     </row>
-    <row r="70">
-      <c r="A70" t="inlineStr">
+    <row r="79">
+      <c r="A79" t="inlineStr">
         <is>
           <t>UPG-82</t>
         </is>
       </c>
-      <c r="B70" t="inlineStr">
+      <c r="B79" t="inlineStr">
         <is>
           <t>执行引擎 S4：ApprovalGroup 双状态机 + EXPIRED + EdgePolicy 失败传播（能力级）</t>
         </is>
       </c>
-      <c r="C70" t="inlineStr">
+      <c r="C79" t="inlineStr">
         <is>
           <t>P1 → ✅ **验收员复验 通过 @2026-09-03**（ACCEPTANCE_LOG §P38：6e9f90e 隔离 worktree——模块 88/0 亲跑[S2/S3 60 零回归+S4 28]+组簿 compute 单桶锁（§P29 教训前置）+**M3 亲杀**[组闸删除→2 红——S3 绕道封死]+M1/M2/M4 采信+S2/S3 零改动辨析+coverage FULL；**达待合→审验员→设计师[合序 71→72→73R1→82]**）
 → ✅ **已合 main @fe8cd45 @2026-09-03**</t>
         </is>
       </c>
-      <c r="D70" t="inlineStr">
+      <c r="D79" t="inlineStr">
         <is>
           <t>📌 **已派单·待认领 @2026-09-03**（派单 `设计师\派单\UPG-82_执行引擎S4_派单_2026-09-03.md`；</t>
         </is>
       </c>
-      <c r="E70" t="inlineStr">
+      <c r="E79" t="inlineStr">
         <is>
           <t>✅**C 完成 @2026-09-03 10:17**（feat/upg82 **6e9f90e** 已 push origin，基底 ma</t>
         </is>
       </c>
-      <c r="F70" t="inlineStr">
+      <c r="F79" t="inlineStr">
         <is>
           <t>✅ **验收员复验 通过 @2026-09-03**（ACCEPTANCE_LOG §P38：6e9f90e 隔离 worktree｜模块</t>
         </is>
       </c>
-      <c r="G70" t="inlineStr">
+      <c r="G79" t="inlineStr">
         <is>
           <t>✅ **已合 main @fe8cd45 @2026-09-03**（设计师B：验收 §P38+审验 confirmed 达待合后｜reba</t>
         </is>
       </c>
-      <c r="H70" t="inlineStr">
+      <c r="H79" t="inlineStr">
         <is>
           <t>设计师\派单\UPG-82_执行引擎S4_派单_2026-09-03.md</t>
         </is>
       </c>
-      <c r="I70" t="inlineStr">
+      <c r="I79" t="inlineStr">
         <is>
           <t>DEL-UPG82-20260903-001</t>
         </is>
       </c>
     </row>
-    <row r="71">
-      <c r="A71" t="inlineStr">
+    <row r="80">
+      <c r="A80" t="inlineStr">
         <is>
           <t>UPG-83</t>
         </is>
       </c>
-      <c r="B71" t="inlineStr">
+      <c r="B80" t="inlineStr">
         <is>
           <t>CODE 模式 tool.call 受控通道（SDK 弃 curl 匝道）</t>
         </is>
       </c>
-      <c r="C71" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D71" t="inlineStr">
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D80" t="inlineStr">
         <is>
           <t>拍板「只要两种模式：经典+极简，极简只是画面极简不阉割能力」｜5→2 模式收敛转 UPG-84：code 模式退役，本单修复对象消失，根因消</t>
         </is>
       </c>
-      <c r="E71" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F71" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G71" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H71" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I71" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-    </row>
-    <row r="72">
-      <c r="A72" t="inlineStr">
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F80" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G80" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H80" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I80" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
         <is>
           <t>UPG-84</t>
         </is>
       </c>
-      <c r="B72" t="inlineStr">
+      <c r="B81" t="inlineStr">
         <is>
           <t>模式收敛 5→2（工具面去模式化 + SDK 匝道段删除）</t>
         </is>
       </c>
-      <c r="C72" t="inlineStr">
+      <c r="C81" t="inlineStr">
         <is>
           <t>P1 → ✅ **验收员复验 带缺陷通过 @2026-09-03**（ACCEPTANCE_LOG §P35：e95472f 隔离 worktree——全量 724/2/1 亲跑一致[UPG-81 未开工口径成立]+Upg84ModeConverge 6 锚全绿+五模式零残留[ToolSdkGenerator 部分保留=tool.help 零缩减待追认]+set_mode 全链路退役+生成器重生成同步+**变异锚① 亲杀**+快速/深思 reasoning 绑模式；用户平板 L3 留用户；**达待合→审验员→设计师**）
 → **依据**：五模式循环（both/code/native/hardware/causal，E3 时代工程产物）从用户面退役——工具面固定全量 both；code 模式退役 → UPG-83（tool.call 补丁单）取消（根因消除优于补丁）；两态开关「经典⇄极简」归极简批阶段 1（送审稿入口决策点，不在本单）
@@ -3782,241 +4205,241 @@
 → ✅ **C 交付 @2026-09-03 08:33**</t>
         </is>
       </c>
-      <c r="D72" t="inlineStr">
+      <c r="D81" t="inlineStr">
         <is>
           <t>📌 **已派单·待认领 @2026-09-03**（用户拍板「只要两种模式：经典+极简，极简只是画面极简不能阉割能力」；派单 `设计师\派</t>
         </is>
       </c>
-      <c r="E72" t="inlineStr">
+      <c r="E81" t="inlineStr">
         <is>
           <t>✅ **C 交付 @2026-09-03 08:33**（程序员 Claude/wmw0027，commit e95472f @feat/u</t>
         </is>
       </c>
-      <c r="F72" t="inlineStr">
+      <c r="F81" t="inlineStr">
         <is>
           <t>✅ **验收员复验+审验 通过 @2026-09-03**（ACCEPTANCE_LOG §P35 + 审验 confirmed：e9547</t>
         </is>
       </c>
-      <c r="G72" t="inlineStr">
+      <c r="G81" t="inlineStr">
         <is>
           <t>✅ **已合 main @8647ee9 @2026-09-03**（设计师B：ff-only 合入+**已 push origin/mai</t>
         </is>
       </c>
-      <c r="H72" t="inlineStr">
+      <c r="H81" t="inlineStr">
         <is>
           <t>设计师\派单\UPG-84_模式收敛_派单_2026-09-03.md</t>
         </is>
       </c>
-      <c r="I72" t="inlineStr">
+      <c r="I81" t="inlineStr">
         <is>
           <t>DEL-UPG84-20260903-001</t>
         </is>
       </c>
     </row>
-    <row r="73">
-      <c r="A73" t="inlineStr">
+    <row r="82">
+      <c r="A82" t="inlineStr">
         <is>
           <t>UPG-85</t>
         </is>
       </c>
-      <c r="B73" t="inlineStr">
+      <c r="B82" t="inlineStr">
         <is>
           <t>预审单 removeAll 缺陷修复（同 tool 多步骤被误移除）</t>
         </is>
       </c>
-      <c r="C73" t="inlineStr">
+      <c r="C82" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
-      <c r="D73" t="inlineStr">
+      <c r="D82" t="inlineStr">
         <is>
           <t>📌 **已派单·待认领 @2026-09-03**（派单 `设计师\派单\UPG-85_预审单removeAll缺陷修复_派单_2026-</t>
         </is>
       </c>
-      <c r="E73" t="inlineStr">
+      <c r="E82" t="inlineStr">
         <is>
           <t>✅**C 完成 @2026-09-03 17:05**（feat/upg85 **8609d69** 已 push origin，基底 ma</t>
         </is>
       </c>
-      <c r="F73" t="inlineStr">
+      <c r="F82" t="inlineStr">
         <is>
           <t>✅ **已闭环（补登 @2026-09-05）**（审验员 09-05 核实：本单实物=8609d69 预审单 removeAll 修复[r</t>
         </is>
       </c>
-      <c r="G73" t="inlineStr">
+      <c r="G82" t="inlineStr">
         <is>
           <t>✅ **已合 main @ad1e0a8 @2026-09-03**（设计师B：rebase fab7d29 零冲突+patch-id 37</t>
         </is>
       </c>
-      <c r="H73" t="inlineStr">
+      <c r="H82" t="inlineStr">
         <is>
           <t>设计师\派单\UPG-85_预审单removeAll缺陷修复_派单_2026-09-03.md</t>
         </is>
       </c>
-      <c r="I73" t="inlineStr">
+      <c r="I82" t="inlineStr">
         <is>
           <t>DEL-UPG85-20260903-001</t>
         </is>
       </c>
     </row>
-    <row r="74">
-      <c r="A74" t="inlineStr">
+    <row r="83">
+      <c r="A83" t="inlineStr">
         <is>
           <t>UPG-86</t>
         </is>
       </c>
-      <c r="B74" t="inlineStr">
+      <c r="B83" t="inlineStr">
         <is>
           <t>manifest 治理（存量补齐 + 审验.py 机器可验性强化）</t>
         </is>
       </c>
-      <c r="C74" t="inlineStr">
+      <c r="C83" t="inlineStr">
         <is>
           <t>P2
 → ✅ **已闭环 @2026-09-03**（验收+审验通过：--manifest-self-test PASS 4/4+存量治理亲验[82/85/87 重验 ok:True 三连+缺失显式 missing 不造假]+双挂账销项落表；工单系统侧无合 main 对象）
 → 🆕 **已认领 @2026-09-03 18:50**</t>
         </is>
       </c>
-      <c r="D74" t="inlineStr">
+      <c r="D83" t="inlineStr">
         <is>
           <t>📌 **已派单·待认领 @2026-09-03**（派单 `设计师\派单\UPG-86_manifest治理_派单_2026-09-03.</t>
         </is>
       </c>
-      <c r="E74" t="inlineStr">
+      <c r="E83" t="inlineStr">
         <is>
           <t>✅**C 完成 @2026-09-03 19:0x**（治理 commit **13434e7**[工单系统仓库]；三件全交：①**审验.p</t>
         </is>
       </c>
-      <c r="F74" t="inlineStr">
+      <c r="F83" t="inlineStr">
         <is>
           <t>✅ **已闭环 @2026-09-03**（验收+审验通过：--manifest-self-test PASS 4/4+存量治理亲验[82/</t>
         </is>
       </c>
-      <c r="G74" t="inlineStr">
+      <c r="G83" t="inlineStr">
         <is>
           <t>合 main对象）</t>
         </is>
       </c>
-      <c r="H74" t="inlineStr">
+      <c r="H83" t="inlineStr">
         <is>
           <t>设计师\派单\UPG-86_manifest治理_派单_2026-09-03.md</t>
         </is>
       </c>
-      <c r="I74" t="inlineStr">
+      <c r="I83" t="inlineStr">
         <is>
           <t>DEL-UPG86-20260903-001</t>
         </is>
       </c>
     </row>
-    <row r="75">
-      <c r="A75" t="inlineStr">
+    <row r="84">
+      <c r="A84" t="inlineStr">
         <is>
           <t>UPG-87</t>
         </is>
       </c>
-      <c r="B75" t="inlineStr">
+      <c r="B84" t="inlineStr">
         <is>
           <t>内置包启停真实生效（宿主工具组纳入 builtin 包机制）</t>
         </is>
       </c>
-      <c r="C75" t="inlineStr">
+      <c r="C84" t="inlineStr">
         <is>
           <t>P1 → ✅ **验收员复验 通过 @2026-09-03**（ACCEPTANCE_LOG §P41：fea2fae 隔离 worktree——全量 **741/0/1 亲跑[0 失败基线兑现首单]**+四件核物[三宿主组纳入/hostPackTools 单源/syncHostBuiltinTools 启停链/默认全量]+McpMarketTest 2→5 零回归[挂账-upg41v2 销项]+**变异复杀如实**[M3 机制采信/M1 未复现红采信 XML 口径]；真机启停 UI 走查=验收员持有待办；**达待合→审验员→设计师[verify-hash 终态]**）
 → ✅ **已合 main @fea2fae @2026-09-03**</t>
         </is>
       </c>
-      <c r="D75" t="inlineStr">
+      <c r="D84" t="inlineStr">
         <is>
           <t>📌 **已派单·待认领 @2026-09-03**（设计师B 溯源实证后出卡；派单 `设计师\派单\UPG-87_内置包启停_派单_202</t>
         </is>
       </c>
-      <c r="E75" t="inlineStr">
+      <c r="E84" t="inlineStr">
         <is>
           <t>✅**C 完成 @2026-09-03 18:4x**（feat/upg87 **fea2fae** 已 push origin，基底 ma</t>
         </is>
       </c>
-      <c r="F75" t="inlineStr">
+      <c r="F84" t="inlineStr">
         <is>
           <t>✅ **验收员复验 通过 @2026-09-03**（ACCEPTANCE_LOG §P41：fea2fae 隔离 worktree｜全量</t>
         </is>
       </c>
-      <c r="G75" t="inlineStr">
+      <c r="G84" t="inlineStr">
         <is>
           <t>✅ **已合 main @fea2fae @2026-09-03**（设计师B：验收 §P41+审验 confirmed[变异环 M1/M3</t>
         </is>
       </c>
-      <c r="H75" t="inlineStr">
+      <c r="H84" t="inlineStr">
         <is>
           <t>设计师\派单\UPG-87_内置包启停_派单_2026-09-03.md</t>
         </is>
       </c>
-      <c r="I75" t="inlineStr">
+      <c r="I84" t="inlineStr">
         <is>
           <t>DEL-UPG87-20260903-001</t>
         </is>
       </c>
     </row>
-    <row r="76">
-      <c r="A76" t="inlineStr">
+    <row r="85">
+      <c r="A85" t="inlineStr">
         <is>
           <t>UPG-88</t>
         </is>
       </c>
-      <c r="B76" t="inlineStr">
+      <c r="B85" t="inlineStr">
         <is>
           <t>极简批阶段 1（ASR + 极简主页生产化 + 两态开关点亮 + 快速提示词）</t>
         </is>
       </c>
-      <c r="C76" t="inlineStr">
+      <c r="C85" t="inlineStr">
         <is>
           <t>P1 → ✅ **验收员复验 带缺陷通过 @2026-09-03**（ACCEPTANCE_LOG §P42：43e5756 三提交链隔离 worktree——全量 **748/0/1 亲跑一致**+Upg84ModeConverge 6 锚全绿[契约升级非消音复核]+R1 自纠实锤+**变异复验 5 轮未复现红如实标注**[采信程序员红案]+L2 四场景采信[未独立复跑如实标注]；coverage PARTIAL 裁决位维持[ASR 真人发声]；**达待合→审验员→设计师**）
 → ✅ **已合 main @43e5756 @2026-09-03**</t>
         </is>
       </c>
-      <c r="D76" t="inlineStr">
+      <c r="D85" t="inlineStr">
         <is>
           <t>📌 **已派单·待认领 @2026-09-03**（产品主线；设计文=极简送审稿+用户拍板「两模式/不阉割能力」；派单 `设计师\派单\U</t>
         </is>
       </c>
-      <c r="E76" t="inlineStr">
+      <c r="E85" t="inlineStr">
         <is>
           <t>✅**C 完成 @2026-09-03 23:0x**（feat/upg88 **43e5756** 已 push origin[施工 90</t>
         </is>
       </c>
-      <c r="F76" t="inlineStr">
+      <c r="F85" t="inlineStr">
         <is>
           <t>**用户指示模拟器自测**（ASR 真实语音转写=物理受限转验收员持有｜coverage PARTIAL 设计师裁决位申报在报告 §七）；T</t>
         </is>
       </c>
-      <c r="G76" t="inlineStr">
+      <c r="G85" t="inlineStr">
         <is>
           <t>✅ **已合 main @43e5756 @2026-09-03**（设计师B：验收 §P42+审验 confirmed[契约升级非消音精读</t>
         </is>
       </c>
-      <c r="H76" t="inlineStr">
+      <c r="H85" t="inlineStr">
         <is>
           <t>设计师\派单\UPG-88_极简批阶段1_派单_2026-09-03.md</t>
         </is>
       </c>
-      <c r="I76" t="inlineStr">
+      <c r="I85" t="inlineStr">
         <is>
           <t>DEL-UPG88-20260903-001</t>
         </is>
       </c>
     </row>
-    <row r="77">
-      <c r="A77" t="inlineStr">
+    <row r="86">
+      <c r="A86" t="inlineStr">
         <is>
           <t>UPG-89</t>
         </is>
       </c>
-      <c r="B77" t="inlineStr">
+      <c r="B86" t="inlineStr">
         <is>
           <t>极简呈现引擎（PresentationRegistry + core.js 呈现栈 + Intent Router + Response Splitter + 三骨架）</t>
         </is>
       </c>
-      <c r="C77" t="inlineStr">
+      <c r="C86" t="inlineStr">
         <is>
           <t>P1 → ✅ **验收员复验 带缺陷通过 @2026-09-03**（ACCEPTANCE_LOG §P46：f616b38f 分支头隔离 worktree——bun 12/12 亲跑+JVM 759/0/1 亲跑[AssetsHomeEngineContract 4 锚]+**PV-01 变异亲杀**[2 fail→还原]；锚⑥死变异裁决转设计师[测试有效性非产品缺陷]；homeWeb 接线下批申报一致；L2 七场景持有；**达待合→审验员→设计师**）→ ✅ **审验 confirmed 带缺陷通过 @2026-09-04**（PV-01 亲杀独立复验双红+锚⑥更精确定性=layer 死状态只写不读+四项发现登记）→ ✅ **已合 main @fe258949 @2026-09-04**（设计师B：rebase 254d6caf 零冲突[原链 a51238dd→615f3590→f616b38f 重写成 84d11731→1e90bf44→fe258949——DEL 绑 615f359 漂移随 UPG-92 硬规则处置]+ff-only+push origin/main+verify-hash HASH_OK 闭环；MainActivity 零触碰=UPG-93 防撞兑现；L2 真机七场景[含 ASR⑦]验收员持有维持；锚⑥ layer 死字段删除随批 P3）→ ✅ **P3 尾巴合入 @0aad7980 @2026-09-04**（程序员锚⑥处置收尾：①核实「断言无需重设计——z 数值断言直调 zSnapshot=方案 a 本在链」②删 surface.layer 死字段[core.js 2 行纯删除，diff 核实一致]+DEL 按新硬规则重绑分支头 4fd540a6；设计师轻量通道：diff 精读[仅 2 删行]+rebase main 单提交回放[旧三链 patch-id 自动跳过]+ff-only+push+verify-hash HASH_OK；锚⑥本活实证[决策丢失变异→zSnapshot topKind=content→RED]在案——「审批永远压内容」安全不变量有杀）
 → 🆕 **已认领 @2026-09-04**（程序员 Claude/wmw0027，worktree mov-upg89，branch feat/upg89，基 main 39b17c4[UPG-90 已合]；按 STD-UPG-89-v2 施工：PresentationRegistry 九字段+style_tokens 白名单+core.js 呈现栈[Surface 四类/Transient-Persistent/z 序置顶/docked/Motion Intent 五词]+Intent Router 四路仲裁+Response Splitter 解析隔离+PV-01 词表闸+Danger 白名单+三骨架——8 变异锚+真机七场景[ASR PARTIAL 随本单补验]；**防撞口径确认**：只动 assets/home 呈现面+新增 core.js/Registry，不碰 MainActivity 工具注册区[UPG-93 拆分在途 WIP]）→ ✅**C 完成 @2026-09-04 04:1x**（feat/upg89 **615f359** 已 push origin[第一批 90aee9f→锚⑥升级 615f359]，基 main 39b17c4[UPG-90 已合]；**引擎全栈落地**：①**core.js 呈现引擎核心**[受信样式词汇表七命名空间 21 词 version 1.2 裸词非法+**PV-01** 原始视觉字面量拒收[视觉键名+hex/px/% 递归扫描]+**Danger 白名单**四词越表拒收+**PresentationRegistry** 九字段+style_tokens 壳级白名单+state 治理 candidate/registered/removed 未登记 fail-closed telemetry+**Response Splitter** 双段解析隔离坏块不塌散文+**SurfaceStack** L0-L4 决策置顶浅栈深度 policy 收叠→Recall+**IntentRouter** 四路仲裁 Cancel/Modify/NewTask/Defer 全足迹+**Motion Intent 五词映射**[enter 300/exit 250/expand 200/docked 450/micro 150+M3 easing]+**三骨架 HTML 生成器** offerCard/timelineList/plain 未登记纯文本回落诚实小字——UMD 双态 node/bun 可测] ②**registry_seed.js** 三骨架登记[offerCard.v1/timelineList.v1/plain.v1 registered+壳白名单] ③**home.html 引擎接入**[core.js/registry_seed 装载+呈现栈容器 present-stack+Recall 圆片条+Intent Router 接线 sendText[cancel/defer 拦截]+docked 态 CSS+v1.2 卡面 token 圆角 22/无描边/--card-shadow-lg/caps 10.5·700·.12em/pill 主钮纯黑+prefers-reduced-motion 退化] ④**测试双层**[bun tests/upg89_core.test.mjs **12/12**[逻辑级 8 锚全对应]+JVM 源码锚 AssetsHomeEngineContractTest **4**[Registry 九字段/三道闸/Motion 五词/Splitter 形态]]；**变异 8 锚：7 实杀 RED**[M1 renderRaw 不抛/M2 扫描恒空/M3 词表恒 ok/M4 Danger 恒放行/M5 未登记不回落/M7 仲裁恒 normal/M8 栈深不收叠——全部 bun RED]+**锚⑥死变异暴露→测试有效性升级**[zSnapshot layer-aware 排序+z 数值断言（决策 L3≥30/内容&lt;30）——加强变异仍 NOT-RED 复跑转复验在案 commit 615f359]；全量 **105 套件 759/0/1 全绿**[755[U90]+4 JVM 锚=759]；**逻辑面四场景机制实证**[①底座输入常驻继承 U88/③审批置顶+Danger 红 bun/④仲裁足迹 bun/⑤未登记回落 bun——真机七场景**转验收员持有**[②agent 流接线+⑦ASR 真人发声——如实申报]；**防撞兑现**[MainActivity 零触碰纯 CRLF+UPG-93 工具注册区零交集]；Token 双段零额外轮次+voice_hint 确定性槽/KV 0；coverage_status=**PARTIAL**[JS 引擎逻辑面 FULL[bun 12/12+7 锚实杀]/原生 agent chunk→homeWeb 接线未做=真机批/下批——设计师裁决位申报]；DEL-UPG89-20260904-001[code=**4fd540a6** 锚⑥处置收尾重绑/artifact=ba3d877dad14c566（APK 前 16）/manifest_sha 见案——**按新硬规则分支头重绑 @2026-09-04**（前头 615f359=f616b38f 链已废，本头含 surface.layer 死字段删除+锚⑥ z 数值断言收口）]；报告 DELIVERY_UPG89_2026-09-04.md；**已登记两个表**）——待验收员验收（L1 复核+变异复杀[bun]+真机七场景[含 agent 接线下批]+合后 verify-hash 终态复核）
@@ -4024,193 +4447,193 @@
 → **防撞**：UPG-88 已合 main</t>
         </is>
       </c>
-      <c r="D77" t="inlineStr">
+      <c r="D86" t="inlineStr">
         <is>
           <t>📌 **已派单·待认领 @2026-09-04**（**v2 正式派发**：启动条件齐=尾巴批清完+UPG-88 已合 main 43e5</t>
         </is>
       </c>
-      <c r="E77" t="inlineStr">
+      <c r="E86" t="inlineStr">
         <is>
           <t>✅**C 完成 @2026-09-04 04:1x**（feat/upg89 **615f359** 已 push origin[第一批 9</t>
         </is>
       </c>
-      <c r="F77" t="inlineStr">
+      <c r="F86" t="inlineStr">
         <is>
           <t>✅ **审验 confirmed 带缺陷通过 @2026-09-04**（PV-01 亲杀独立复验双红+锚⑥更精确定性=layer 死状态只</t>
         </is>
       </c>
-      <c r="G77" t="inlineStr">
+      <c r="G86" t="inlineStr">
         <is>
           <t>✅ **已合 main @fe258949 @2026-09-04**（设计师B：rebase 254d6caf 零冲突[原链 a51238</t>
         </is>
       </c>
-      <c r="H77" t="inlineStr">
+      <c r="H86" t="inlineStr">
         <is>
           <t>设计师\派单\UPG-89_极简呈现引擎_派单_2026-09-03.md</t>
         </is>
       </c>
-      <c r="I77" t="inlineStr">
+      <c r="I86" t="inlineStr">
         <is>
           <t>DEL-UPG89-20260904-001</t>
         </is>
       </c>
     </row>
-    <row r="78">
-      <c r="A78" t="inlineStr">
+    <row r="87">
+      <c r="A87" t="inlineStr">
         <is>
           <t>UPG-90</t>
         </is>
       </c>
-      <c r="B78" t="inlineStr">
+      <c r="B87" t="inlineStr">
         <is>
           <t>尾巴批修（S-06 打回项 ②⑧ + C7 基线测试非确定性）</t>
         </is>
       </c>
-      <c r="C78" t="inlineStr">
+      <c r="C87" t="inlineStr">
         <is>
           <t>P2 → ✅ **验收员复验 通过 @2026-09-03**（ACCEPTANCE_LOG §P47：c969b05a 隔离 worktree——全量 **762/0/0 亲跑**[0 失败基线]+ToolsSplitContract 7 锚+9 域拆分+MainActivity 1752 行删减+零行为变化[sha256 双锁]+**M-vault 变异亲杀**[键名变异→3 锚齐红与申报一致→还原；注释式破多行 lambda 编译失败教训三现——拆分类变异用键名/删除式]；冷启动 +5.1%&lt;10%；真机三场景采信；**达待合→审验员→设计师**[阶段 2 后续]）
 → ✅ **已合 main @39b17c4 @2026-09-03**</t>
         </is>
       </c>
-      <c r="D78" t="inlineStr">
+      <c r="D87" t="inlineStr">
         <is>
           <t>📌 **已派单·待认领 @2026-09-03**（尾巴清零批；派单 `设计师\派单\UPG-90_尾巴批修_派单_2026-09-03.</t>
         </is>
       </c>
-      <c r="E78" t="inlineStr">
+      <c r="E87" t="inlineStr">
         <is>
           <t>✅**C 完成 @2026-09-04 00:1x**（feat/upg90 **1845cb7** 已 push origin，基 mai</t>
         </is>
       </c>
-      <c r="F78" t="inlineStr">
+      <c r="F87" t="inlineStr">
         <is>
           <t>✅ **验收员复验 通过 @2026-09-03**（ACCEPTANCE_LOG §P47：c969b05a 隔离 worktree｜全量</t>
         </is>
       </c>
-      <c r="G78" t="inlineStr">
+      <c r="G87" t="inlineStr">
         <is>
           <t>✅ **已合 main @39b17c4 @2026-09-03**（设计师B：验收 §P43+审验 confirmed 达待合后｜reba</t>
         </is>
       </c>
-      <c r="H78" t="inlineStr">
+      <c r="H87" t="inlineStr">
         <is>
           <t>设计师\派单\UPG-90_尾巴批修_派单_2026-09-03.md</t>
         </is>
       </c>
-      <c r="I78" t="inlineStr">
+      <c r="I87" t="inlineStr">
         <is>
           <t>DEL-UPG90-20260903-001</t>
         </is>
       </c>
     </row>
-    <row r="79">
-      <c r="A79" t="inlineStr">
+    <row r="88">
+      <c r="A88" t="inlineStr">
         <is>
           <t>UPG-91</t>
         </is>
       </c>
-      <c r="B79" t="inlineStr">
+      <c r="B88" t="inlineStr">
         <is>
           <t>我的资产页注册制重排（tab 导航+二级收缩裸列表+点值脱敏+诚实空态+假数据回落删除+令牌迁移）</t>
         </is>
       </c>
-      <c r="C79" t="inlineStr">
+      <c r="C88" t="inlineStr">
         <is>
           <t>P2 → ✅ **验收员复验 带缺陷通过 @2026-09-03**（ACCEPTANCE_LOG §P44：4dc19e7 三提交链隔离 worktree——全量 **752/0/1 亲跑一致**+demoBridge 假数据零残留 grep[红线 18 同族根除]+锚④强化实录复核+R1 自纠[1C 形态消费恢复]；变异 M4 未复现如实[采信程序员 4/4 XML]；真机五场景持有维持；**达待合→审验员→设计师**）
 → ✅ **已合 main @4dc19e7 @2026-09-03**</t>
         </is>
       </c>
-      <c r="D79" t="inlineStr">
+      <c r="D88" t="inlineStr">
         <is>
           <t>📌 **已派单·待认领 @2026-09-03**（用户实测「体验感很差」→ 四病灶诊断 → 六轮迭代 demo v6 拍板；派单 `设计</t>
         </is>
       </c>
-      <c r="E79" t="inlineStr">
+      <c r="E88" t="inlineStr">
         <is>
           <t>✅**C 完成 @2026-09-04 01:4x**（feat/upg91 **34a2dda** 已 push origin[远端顶=4</t>
         </is>
       </c>
-      <c r="F79" t="inlineStr">
+      <c r="F88" t="inlineStr">
         <is>
           <t>✅ **验收员复验 带缺陷通过 @2026-09-03**（ACCEPTANCE_LOG §P44：4dc19e7 三提交链隔离 workt</t>
         </is>
       </c>
-      <c r="G79" t="inlineStr">
+      <c r="G88" t="inlineStr">
         <is>
           <t>✅ **已合 main @4dc19e7 @2026-09-03**（设计师B：验收 §P44+审验 confirmed[M4 复杀补强｜验</t>
         </is>
       </c>
-      <c r="H79" t="inlineStr">
+      <c r="H88" t="inlineStr">
         <is>
           <t>设计师\派单\UPG-91_我的资产页重排_派单_2026-09-03.md</t>
         </is>
       </c>
-      <c r="I79" t="inlineStr">
+      <c r="I88" t="inlineStr">
         <is>
           <t>DEL-UPG91-20260904-001</t>
         </is>
       </c>
     </row>
-    <row r="80">
-      <c r="A80" t="inlineStr">
+    <row r="89">
+      <c r="A89" t="inlineStr">
         <is>
           <t>UPG-92</t>
         </is>
       </c>
-      <c r="B80" t="inlineStr">
+      <c r="B89" t="inlineStr">
         <is>
           <t>manifest 硬闸化（deliver-gen 源头合规 + 自检内置）</t>
         </is>
       </c>
-      <c r="C80" t="inlineStr">
+      <c r="C89" t="inlineStr">
         <is>
           <t>P1 → ✅ **验收员复验 通过 @2026-09-03**（ACCEPTANCE_LOG §P45：39039ef 工单系统仓隔离 worktree——**deliver-gen --self-test 4/4 亲跑 PASS**[源头合规/硬闸注入红×2 exit=1 残件清除/骨架回归]+硬闸「拒绝产出非警告」机制化——**第六现根因闭环**；DEL-UPG92 狗粮自证；观察转办：sync 锚词表「✅K 完成」代号→设计师；**达待合→设计师**）
 → ✅ **已合 main</t>
         </is>
       </c>
-      <c r="D80" t="inlineStr">
+      <c r="D89" t="inlineStr">
         <is>
           <t>📌 **已派单·待认领 @2026-09-03**（manifest 同族第六现｜红线 23 自检步声称未执行，改机制硬闸；派单 `设计师</t>
         </is>
       </c>
-      <c r="E80" t="inlineStr">
+      <c r="E89" t="inlineStr">
         <is>
           <t>✅**C 完成 @2026-09-04 00:0x**（程序员 Kimi/kimi-cli，feat/upg92 **39039ef** 已</t>
         </is>
       </c>
-      <c r="F80" t="inlineStr">
+      <c r="F89" t="inlineStr">
         <is>
           <t>✅ **验收员复验 通过 @2026-09-03**（ACCEPTANCE_LOG §P45：39039ef 工单系统仓隔离 worktre</t>
         </is>
       </c>
-      <c r="G80" t="inlineStr">
+      <c r="G89" t="inlineStr">
         <is>
           <t>✅ **已合 main（工单系统仓）@beb2777 @2026-09-03**（设计师B：验收 §P45+审验 confirmed 后｜f</t>
         </is>
       </c>
-      <c r="H80" t="inlineStr">
+      <c r="H89" t="inlineStr">
         <is>
           <t>设计师\派单\UPG-92_manifest硬闸化_派单_2026-09-03.md</t>
         </is>
       </c>
-      <c r="I80" t="inlineStr">
+      <c r="I89" t="inlineStr">
         <is>
           <t>DEL-UPG92-20260904-001</t>
         </is>
       </c>
     </row>
-    <row r="81">
-      <c r="A81" t="inlineStr">
+    <row r="90">
+      <c r="A90" t="inlineStr">
         <is>
           <t>UPG-93</t>
         </is>
       </c>
-      <c r="B81" t="inlineStr">
+      <c r="B90" t="inlineStr">
         <is>
           <t>MainActivity 拆分·阶段 1（工具注册面搬移 + 拆分蓝图落档）</t>
         </is>
       </c>
-      <c r="C81" t="inlineStr">
+      <c r="C90" t="inlineStr">
         <is>
           <t>P1
 → 🆕 **已认领 @2026-09-04 01:5x**（程序员 Claude/wmw0027，worktree mov-upg93，branch feat/upg93，基 main 254d6ca[军规 commit 顶]；按派单施工：185 handler 盘点落蓝图+ToolsRegistry 聚合+分域 Registrar 搬移+3 变异锚+测试金字塔——纯搬移零逻辑改动）→ ⚠️**WIP 回滚 @2026-09-04 02:3x**（程序员 C：盘点/口径闭合/提取器基建完成入库[commit 76c91cb：169 注册点三态扫描盘点+9 域归类+185 口径闭合核对]；**搬移实施中途回滚**——三态提取器跑出的 9 域文件存在块边界错位残片[ModelRegistry 循环/obsidian 段等 5-8 处——三方对账未完成]，**不带入半成品**，工作区已还原 7666 行原始态；工程形态已定案=Kotlin 扩展函数分域文件[receiver=this 零改动零持有]，WIP 资产与修复路径在案[upg93-拆分wip 记忆+upg93_inventory.json]）——**重新认领需独立完整会话**（剩余：错位残片三方对账→测试金字塔→3 变异锚→冷启动锚）
@@ -4221,49 +4644,49 @@
 → 🆕 **已认领 @2026-09-04 01:58·重新接管**</t>
         </is>
       </c>
-      <c r="D81" t="inlineStr">
+      <c r="D90" t="inlineStr">
         <is>
           <t>📌 **已派单·待认领 @2026-09-03**（架构图实证「图上分层、代码一锅」｜用户拍板「先解决这个」；派单 `设计师\派单\UPG</t>
         </is>
       </c>
-      <c r="E81" t="inlineStr">
+      <c r="E90" t="inlineStr">
         <is>
           <t>✅**C 完成 @2026-09-04 03:3x**（程序员 Kimi/kimi-cli，feat/upg93 **c969b05a**</t>
         </is>
       </c>
-      <c r="F81" t="inlineStr">
+      <c r="F90" t="inlineStr">
         <is>
           <t>✅ **验收员复验通过（§P47）→ 审验 confirmed 通过 @2026-09-04**（M-vault 键名变异亲杀 3 锚齐红独</t>
         </is>
       </c>
-      <c r="G81" t="inlineStr">
+      <c r="G90" t="inlineStr">
         <is>
           <t>✅ **已合 main @3315bff0 @2026-09-04**（设计师B：rebase 0aad7980 零冲突[c969b05a→</t>
         </is>
       </c>
-      <c r="H81" t="inlineStr">
+      <c r="H90" t="inlineStr">
         <is>
           <t>设计师\派单\UPG-93_MainActivity拆分阶段1_派单_2026-09-03.md</t>
         </is>
       </c>
-      <c r="I81" t="inlineStr">
+      <c r="I90" t="inlineStr">
         <is>
           <t>DEL-UPG93-20260904-001</t>
         </is>
       </c>
     </row>
-    <row r="82">
-      <c r="A82" t="inlineStr">
+    <row r="91">
+      <c r="A91" t="inlineStr">
         <is>
           <t>UPG-94</t>
         </is>
       </c>
-      <c r="B82" t="inlineStr">
+      <c r="B91" t="inlineStr">
         <is>
           <t>极简主页真机观感修复（dock 隐藏 + logo 去框去影 + hint 删除 + 发送钮归 token）</t>
         </is>
       </c>
-      <c r="C82" t="inlineStr">
+      <c r="C91" t="inlineStr">
         <is>
           <t>P1 → ✅ **验收员复验 带缺陷通过 @2026-09-03**（ACCEPTANCE_LOG §P48：分支头 25f73fe0[申报 746b20ec≠分支头二现]隔离 worktree——全量 763/0/1 亲跑一致+契约锚 4/4+**M1 删除式亲杀**[failures=1→还原；注释式免疫四现终纳]+四件观感修复核物；**P3×2：U89 引擎恢复自纠未申报**[透明度义务]+logo 168px 追加后截图未更新；**达待合→审验员→设计师**）→ ✅ **审验 confirmed 带缺陷通过 @2026-09-04**（四件坐实+U89 恢复自纠亲核正确完整+四项发现登记）
 → ⚠️ **WIP 回滚 @2026-09-04**（UPG-98 拆分批②市场面——程序员 C：7 块搬移+13 提升+MarketTools 恢复完成[compileDebugKotlin EXIT=0]；**但 5 个测试失败**[锚定面迁移问题——HostBuiltin 2+ToolMeta 2+SceneWiring 1——非产品缺陷]；**toolFaceSrc 加 market/ 联合读源+MarketTools.kt 恢复 ac7495fb 版已 commit dff0ba8a/push**——**实施转独立会话**（锚定面迁移第二批+全量验证+冷启动锚+真机冒烟——上下文预算耗尽不带入半成品）；WIP 资产在案[upg98-拆分批2市场面交付记忆]）——**重新认领需独立完整会话**→ ✅ **已合 main @806bb01c @2026-09-04**（设计师B：rebase 3315bff0 三提交重写[25f73fe0→806bb01c——MainActivity 与 93 双改不同区域自动合并 clean]+ff-only+push+verify-hash HASH_OK；**设计师追加项验收缺口实录**：seed 合并进 engine.registry+timelineList 骨架 CSS 两项[2026-09-04 设计师裁决并 94 随批]未随本单落地——转出至 UPG-96 范围[接线单前置一件]，STD-96 追加说明区已注记；4 项发现裁决见问题区）
@@ -4272,49 +4695,49 @@
 → **防撞**：MainActivity 只动 applyPresentationMode/dock 字段化</t>
         </is>
       </c>
-      <c r="D82" t="inlineStr">
+      <c r="D91" t="inlineStr">
         <is>
           <t>📌 **已派单·待认领 @2026-09-04**（用户真机实测踩中[2026-09-04 03:27 包]：极简态经典 dock 飘顶[</t>
         </is>
       </c>
-      <c r="E82" t="inlineStr">
+      <c r="E91" t="inlineStr">
         <is>
           <t>🆕 **已认领 @2026-09-04**（程序员 Claude/wmw0027，worktree mov-upg94，branch fe</t>
         </is>
       </c>
-      <c r="F82" t="inlineStr">
+      <c r="F91" t="inlineStr">
         <is>
           <t>✅ **审验 confirmed 带缺陷通过 @2026-09-04**（四件坐实+U89 恢复自纠亲核正确完整+四项发现登记）</t>
         </is>
       </c>
-      <c r="G82" t="inlineStr">
+      <c r="G91" t="inlineStr">
         <is>
           <t>✅ **已合 main @806bb01c @2026-09-04**（设计师B：rebase 3315bff0 三提交重写[25f73fe</t>
         </is>
       </c>
-      <c r="H82" t="inlineStr">
+      <c r="H91" t="inlineStr">
         <is>
           <t>设计师\派单\UPG-94_极简主页真机观感修复_派单_2026-09-04.md</t>
         </is>
       </c>
-      <c r="I82" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-    </row>
-    <row r="83">
-      <c r="A83" t="inlineStr">
+      <c r="I91" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
         <is>
           <t>UPG-95</t>
         </is>
       </c>
-      <c r="B83" t="inlineStr">
+      <c r="B92" t="inlineStr">
         <is>
           <t>个性化槽位选择（care profile 提炼 + 可选槽池 + LLM 编辑层 + ticketCard/rideCard 骨架落地）</t>
         </is>
       </c>
-      <c r="C83" t="inlineStr">
+      <c r="C92" t="inlineStr">
         <is>
           <t>P1 → ✅ **验收员复验 通过 @2026-09-04**（ACCEPTANCE_LOG §P49：979bf6bf 三批隔离 worktree——**bun 18/18 亲跑**+全量 **786/0/1 亲跑**[Care 双类 20 用例]+**M-11 变异亲杀**[敏感闸放行→红→还原]+编辑层接线[设计师裁决已接]；其余 3 锚采信；L2 出卡走查持有；**达待合→审验员→设计师**）→ ✅ **审验 confirmed 通过 @2026-09-04**（bun 18/18+全量 786/0/1 双亲跑+M-11 敏感闸亲杀独立复验+DEL 绑定无漂移正面记录[三连回潮后首单做对]）→ ✅ **已合 main @ac7495fb @2026-09-04**（设计师B：rebase 806bb01c 人工解真冲突 2 处[index.html CSS 段取 main 位置+并入 95 amenities/route/driver/pref-chip 装载块+顺带补回 94 恢复时漏网的 docked 态两条 CSS]+解后复跑闸：bun 12+6 全绿+全量 **790/0/1** 绿→ff-only+push+verify-hash HASH_OK；3 项发现裁决见问题区；持有项=L2 出卡 CDP 走查[随 96]+ASR PARTIAL[96 场景⑦]） → ✅ **验收员复验 带缺陷通过 @2026-09-03**（ACCEPTANCE_LOG §P50：cdf769a9 隔离 worktree——全量 **775/0/1 亲跑一致**+**HomeDeliveryContractTest 5/5 亲跑确认**[homeWeb 接线契约落位——UPI-89/95 遗留闭环]+红线/诚实申报复核；**M2 复杀 3 式未复现如实标注**[多行 evaluateJavascript 适配成本超阈值——采信程序员 XML]+L2 模拟器环境阻塞登记；**达待合→审验员→设计师**）
 → 🆕 **已认领 @2026-09-04**（程序员 Claude/wmw0027，worktree mov-upg95，branch feat/upg95，基 main 3315bff0[含 UPG-93 拆分]；施工：提炼层六域规则扩展（hotel/food/rail/ride/travel/shopping 纯函数）+offerCard amenities 槽（≤3）+ticketCard/rideCard candidate 登记+编辑层提示词节[全量事实×画像→槽池内选择；标签注入原文不进]——种子集 11 断言+4 变异锚；与 UPG-94 同 index.html 面按裁决串行）
@@ -4322,96 +4745,96 @@
 → **复用**：UPG-51 提炼器扩展点 + UPG-89 引擎/Registry + UPG-05 基因红线</t>
         </is>
       </c>
-      <c r="D83" t="inlineStr">
+      <c r="D92" t="inlineStr">
         <is>
           <t>📌 **已派单·待认领 @2026-09-04**（用户拍板方向「商户信息尽量全+用户侧个性化显示」；设计口径=v1.2 增补附录 B[三</t>
         </is>
       </c>
-      <c r="E83" t="inlineStr">
+      <c r="E92" t="inlineStr">
         <is>
           <t>🆕 **已认领 @2026-09-04**（程序员 Claude/wmw0027，worktree mov-upg95，branch fe</t>
         </is>
       </c>
-      <c r="F83" t="inlineStr">
+      <c r="F92" t="inlineStr">
         <is>
           <t>✅ **审验 confirmed 通过 @2026-09-04**（bun 18/18+全量 786/0/1 双亲跑+M-11 敏感闸亲杀独</t>
         </is>
       </c>
-      <c r="G83" t="inlineStr">
+      <c r="G92" t="inlineStr">
         <is>
           <t>✅ **已合 main @ac7495fb @2026-09-04**（设计师B：rebase 806bb01c 人工解真冲突 2 处[in</t>
         </is>
       </c>
-      <c r="H83" t="inlineStr">
+      <c r="H92" t="inlineStr">
         <is>
           <t>设计师\派单\UPG-95_个性化槽位选择_派单_2026-09-04.md</t>
         </is>
       </c>
-      <c r="I83" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-    </row>
-    <row r="84">
-      <c r="A84" t="inlineStr">
+      <c r="I92" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
         <is>
           <t>UPG-96</t>
         </is>
       </c>
-      <c r="B84" t="inlineStr">
+      <c r="B93" t="inlineStr">
         <is>
           <t>homeWeb 呈现回路接线（极简发送不回落 + LLM 回复回流出卡 + 真机批收口）</t>
         </is>
       </c>
-      <c r="C84" t="inlineStr">
+      <c r="C93" t="inlineStr">
         <is>
           <t>P1 → ✅ **验收员复验 带缺陷通过 @2026-09-04**</t>
         </is>
       </c>
-      <c r="D84" t="inlineStr">
+      <c r="D93" t="inlineStr">
         <is>
           <t>裁决位]；DEL-UPG96-20260904-001[code=cdf769a9/artifact=04f48903/manifest_s</t>
         </is>
       </c>
-      <c r="E84" t="inlineStr">
+      <c r="E93" t="inlineStr">
         <is>
           <t>✅**C 完成 @2026-09-04**（feat/upg96 **cdf769a9** 已 push origin[远端顶；基 main</t>
         </is>
       </c>
-      <c r="F84" t="inlineStr">
+      <c r="F93" t="inlineStr">
         <is>
           <t>✅ **审验 通过 @2026-09-04**（integrity_review=confirmed：与 §P50 一致，变异环比验收员更深</t>
         </is>
       </c>
-      <c r="G84" t="inlineStr">
+      <c r="G93" t="inlineStr">
         <is>
           <t>✅ 已合 main @6dcfbac9（feat/upg96 cdf769a9 合入+已 push；rebase ac7495fb 零冲突实</t>
         </is>
       </c>
-      <c r="H84" t="inlineStr">
+      <c r="H93" t="inlineStr">
         <is>
           <t>设计师\派单\UPG-96_homeWeb呈现回路接线_派单_2026-09-04.md</t>
         </is>
       </c>
-      <c r="I84" t="inlineStr">
+      <c r="I93" t="inlineStr">
         <is>
           <t>DEL-UPG96-20260904-001</t>
         </is>
       </c>
     </row>
-    <row r="85">
-      <c r="A85" t="inlineStr">
+    <row r="94">
+      <c r="A94" t="inlineStr">
         <is>
           <t>UPG-97</t>
         </is>
       </c>
-      <c r="B85" t="inlineStr">
+      <c r="B94" t="inlineStr">
         <is>
           <t>侧边栏工作台三入口接线（我的记忆/我的资产/我的能力）+ comingSoon 兜底可见性</t>
         </is>
       </c>
-      <c r="C85" t="inlineStr">
+      <c r="C94" t="inlineStr">
         <is>
           <t>P1 → ✅ **验收员复验 带缺陷通过 @2026-09-04**（ACCEPTANCE_LOG §P51：9010075d 工单系统仓隔离 worktree——全量 794/0/0 亲跑一致+**变异双锚亲杀**[分派锚 failures=2/兜底锚 failures=1→还原]+openBuiltin 三 case+comingSoon showDialog+i18n 双字典；**L2 真机四点验实证**[市场/资产/能力/订单]+**我的记忆行 5556 未呈现疑点转办**[平板五点验过——澄清后终判]；**达待合→审验员→设计师**）
 → **防撞**：纯前端单（mov-vue 源+产物同步）；MainActivity/tools 零行；与 95/96 零交集
@@ -4420,49 +4843,49 @@
 → ✅ **已合 main @04ca51ab</t>
         </is>
       </c>
-      <c r="D85" t="inlineStr">
+      <c r="D94" t="inlineStr">
         <is>
           <t>📌 **已派单·待认领 @2026-09-04**（用户真机报障「侧边栏有的按钮失灵」→ 设计师 adb 实测复现+根因定位：Sideba</t>
         </is>
       </c>
-      <c r="E85" t="inlineStr">
+      <c r="E94" t="inlineStr">
         <is>
           <t>✅**C 完成 @2026-09-04 06:5x**（程序员 Kimi/kimi-cli，feat/upg97 **9010075d**</t>
         </is>
       </c>
-      <c r="F85" t="inlineStr">
+      <c r="F94" t="inlineStr">
         <is>
           <t>✅ **验收员复验 带缺陷通过 @2026-09-04**（ACCEPTANCE_LOG §P51：9010075d 工单系统仓隔离 wor</t>
         </is>
       </c>
-      <c r="G85" t="inlineStr">
+      <c r="G94" t="inlineStr">
         <is>
           <t>✅ **已合 main @04ca51ab（2026-09-04 设计师合入）**：rebase origin/main 6dcfbac9</t>
         </is>
       </c>
-      <c r="H85" t="inlineStr">
+      <c r="H94" t="inlineStr">
         <is>
           <t>设计师\派单\UPG-97_侧边栏三入口接线_派单_2026-09-04.md</t>
         </is>
       </c>
-      <c r="I85" t="inlineStr">
+      <c r="I94" t="inlineStr">
         <is>
           <t>DEL-UPG97-20260904-001</t>
         </is>
       </c>
     </row>
-    <row r="86">
-      <c r="A86" t="inlineStr">
+    <row r="95">
+      <c r="A95" t="inlineStr">
         <is>
           <t>UPG-98</t>
         </is>
       </c>
-      <c r="B86" t="inlineStr">
+      <c r="B95" t="inlineStr">
         <is>
           <t>MainActivity 拆分·批② 市场面搬移（→ market/ 模块）</t>
         </is>
       </c>
-      <c r="C86" t="inlineStr">
+      <c r="C95" t="inlineStr">
         <is>
           <t>P1 → ❌ **验收员打回 @2026-09-03**（ACCEPTANCE_LOG §P51b：**P1 提交版测试文件编译不过**——d96ade5d HostBuiltinPackContractTest mainSrc() 裸换行截断字符串→compileDebugUnitTestKotlin FAILED→全量在提交版无法执行；对照实锤：程序员 worktree 同路径=正确版未提交——**提交版≠验证版实锤**；七块搬移结构核过[工作区读源+MarketTools.kt 恢复 U93 遗漏自查]；修=工作区正确版 commit+新 commit 交付+DEL 重绑+R1 全新检出复验；**打回→程序员**） → ⚠️ **§P51c 中间态核验 @2026-09-03**（ACCEPTANCE_LOG 补记：dff0ba8a mainSrc 修复实锤[:27 单行]采纳 §P51b；全量 795/6/1——4 类失败定性=**锚定面迁移未完成**[HostBuiltin seg 锚失效/MarketSplit 集合缺元素/ToolMeta internal 锚未更新/ToolsSplit 1 红——非产品缺陷]；**维持打回（WIP）**——锚定面迁移完成（0 失败）再交 R1 复验） → 📌 **二次 WIP 如实申报处置 @2026-09-03**（脚本自动化搬移失败如实[fun 声明复杂度四条根因入册]——工作区还原 04ca51ab；**验收员核出申报不实一项**：6 文件 D 残留[gen93/scan93b/mut93 等 UPG-93 方法论资产被工作区删除未提交]——已代为恢复[git checkout，资产保全]；UPG-98 状态=**待重新认领·人工逐块搬移路径**[程序员建议：IDE 重构或手工 copy-paste 每块编译一次，30 分钟级]；工作树现状=feat/upg98@04ca51ab 干净） → ✅ **交付·待验收 @2026-09-04**（程序员重做完成[用户直派]：cherry-pick 上轮人工搬移 2787b73a[编译实证过的人工件非脚本]+锚定面迁移全收口=4b279e0a+d11509cc——全量 804/0/1（112 套件 --rerun-tasks）+3 变异锚亲杀红绿闭环[保真点名 buildLocalOverview/名单多挂点名 zzMutant/唯一写点点名 syncBuiltinPackTools]+冷启动双侧 5 次中位 940→932ms（Δ-0.9% 在带内）+真机三场景全过[市场页渲染/启停 185↔172 精确-13/logcat 双行/market.status 直呼]+assembleDebug 绿+Token/KV 0/0；**DEL-UPG98-001 绑分支头 d11509cc**（红线 23 推进=重绑）；manifest=deliver-gen 硬闸产出 ok:True[standard_id 内嵌 sha 交叉校验过]；报告 `程序员\交付报告\DELIVERY_UPG98_2026-09-04.md`；R1 复验→审验员→设计师） → ✅ **R1 复验 通过 @2026-09-04**（ACCEPTANCE_LOG §P52：d11509cc 全新检出 **804/0/1 亲跑终验**[P1 提交版编译不过修复闭环]+MarketSplitContract 5 锚全绿[搬移保真契约锁]+变异 3 锚采信如实[验收员注入 3 轮未达真红——XML+契约双证采信]+L2 真机三场景采信[模拟器四度下线环境阻塞登记]；两观察转办[isAppVisible 不稳定/registry 依赖]；**达待合→审验员→设计师**） → ✅ **审验 confirmed 通过 @2026-09-04**（审验员：从零编译 804/0/0+1 跳过亲跑+变异采信升级亲杀[KDoc 改字→保真锚真红]+拆前 sha 独立抽查=冻结值+问题区 3 项） → ✅ **已合 main @d11509cc @2026-09-04**（04ca51ab→d11509cc 直接快进零冲突，verify-hash 通过；问题区 3 项裁决落档[isAppVisible 呈现通道缺口升级 P2 入审批收口议题/registry 依赖挂账残留面登记/3 函数 public 豁免注记入债务清单]；里程碑：上帝文件 7666→6016→5929 行；批③页面桥待派）
 → **范围**：市场总览区（buildLocalOverview/启停/安装投影）→ market/ 模块；纯搬移零逻辑改动；保真锚=块归一化 sha256 前后全等
@@ -4470,192 +4893,192 @@
 → 🆕 **已认领 @2026-09-04 07:18**</t>
         </is>
       </c>
-      <c r="D86" t="inlineStr">
+      <c r="D95" t="inlineStr">
         <is>
           <t>📌 **已派单·待认领 @2026-09-04**（拆分主线批②/共 8 批｜串行纪律：一批一派合后再基[UPG-95 真冲突实证后立]；</t>
         </is>
       </c>
-      <c r="E86" t="inlineStr">
+      <c r="E95" t="inlineStr">
         <is>
           <t>🆕 **已认领 @2026-09-04 07:18**（程序员 C/Claude-wmw0027，worktree mov-upg98，b</t>
         </is>
       </c>
-      <c r="F86" t="inlineStr">
+      <c r="F95" t="inlineStr">
         <is>
           <t>✅ **审验 confirmed 通过 @2026-09-04**（审验员：从零编译 804/0/0+1 跳过亲跑+变异采信升级亲杀[KDo</t>
         </is>
       </c>
-      <c r="G86" t="inlineStr">
+      <c r="G95" t="inlineStr">
         <is>
           <t>✅ **已合 main @d11509cc @2026-09-04**（04ca51ab→d11509cc 直接快进零冲突，verify-h</t>
         </is>
       </c>
-      <c r="H86" t="inlineStr">
+      <c r="H95" t="inlineStr">
         <is>
           <t>设计师\派单\UPG-98_MainActivity拆分批2市场面_派单_2026-09-04.md</t>
         </is>
       </c>
-      <c r="I86" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-    </row>
-    <row r="87">
-      <c r="A87" t="inlineStr">
+      <c r="I95" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
         <is>
           <t>UPG-99</t>
         </is>
       </c>
-      <c r="B87" t="inlineStr">
+      <c r="B96" t="inlineStr">
         <is>
           <t>工单系统工具链硬闸批（DEL 分支头校验 + standard_id 交叉校验 + 报告模板强制段 + 红线 23 落规）</t>
         </is>
       </c>
-      <c r="C87" t="inlineStr">
+      <c r="C96" t="inlineStr">
         <is>
           <t>P2
 → **范围**：sync-orders DEL==分支头校验 / 审验.py standard_id 交叉校验 / deliver-gen 模板强制段 / 红线 23 两条明文
 → **纪律**：既有闸零回归；报错人话化；改库卡先备份；sync 后 --check diff=0</t>
         </is>
       </c>
-      <c r="D87" t="inlineStr">
+      <c r="D96" t="inlineStr">
         <is>
           <t>✅ **设计师直修完成 @2026-09-04**（用户拍板「你自己修吧，不搞工单」｜不走流转流程，设计师直接落地四件：①deliver-g</t>
         </is>
       </c>
-      <c r="E87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F87" t="inlineStr">
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F96" t="inlineStr">
         <is>
           <t>**范围**：sync-orders DEL==分支头校验 / 审验.py standard_id 交叉校验 / deliver-gen 模</t>
         </is>
       </c>
-      <c r="G87" t="inlineStr">
+      <c r="G96" t="inlineStr">
         <is>
           <t>已合 main@hash」在祖先链/存量 cherry-pick 卡豁免/显式豁免跳过]｜首跑即抓 7 条存量异常全归因[5 存量豁免+1</t>
         </is>
       </c>
-      <c r="H87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-    </row>
-    <row r="88">
-      <c r="A88" t="inlineStr">
+      <c r="H96" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I96" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
         <is>
           <t>UPG-100</t>
         </is>
       </c>
-      <c r="B88" t="inlineStr">
+      <c r="B97" t="inlineStr">
         <is>
           <t>锚②半弱锚升级（count/match 组合断言）</t>
         </is>
       </c>
-      <c r="C88" t="inlineStr">
+      <c r="C97" t="inlineStr">
         <is>
           <t>P2</t>
         </is>
       </c>
-      <c r="D88" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E88" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F88" t="inlineStr">
+      <c r="D97" t="inlineStr">
+        <is>
+          <t>📌 已派单（用户直接外派）</t>
+        </is>
+      </c>
+      <c r="E97" t="inlineStr">
+        <is>
+          <t>✅ C 完成 @2026-09-05（kimi-cli，a63b7088——锚②升级 count/match；待验收）</t>
+        </is>
+      </c>
+      <c r="F97" t="inlineStr">
         <is>
           <t>📌 已立卡·待派 ⏳ @2026-09-04（UPG-96 审验发现项①转正：contains 组合锚对单点破坏免疫）｜ 待派单</t>
         </is>
       </c>
-      <c r="G88" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H88" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I88" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-    </row>
-    <row r="89">
-      <c r="A89" t="inlineStr">
+      <c r="G97" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H97" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I97" t="inlineStr">
+        <is>
+          <t>DEL-UPG100-20260905-001</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
         <is>
           <t>UPG-101</t>
         </is>
       </c>
-      <c r="B89" t="inlineStr">
+      <c r="B98" t="inlineStr">
         <is>
           <t>侧边栏默认插件种子清单（「我的记忆」入口是否纳入 defaults）</t>
         </is>
       </c>
-      <c r="C89" t="inlineStr">
+      <c r="C98" t="inlineStr">
         <is>
           <t>P3</t>
         </is>
       </c>
-      <c r="D89" t="inlineStr">
+      <c r="D98" t="inlineStr">
         <is>
           <t>拍板@2026-09-04（UPG-97 合 main 随批</t>
         </is>
       </c>
-      <c r="E89" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F89" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G89" t="inlineStr">
+      <c r="E98" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F98" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G98" t="inlineStr">
         <is>
           <t>📌 挂单·待用户拍板 @2026-09-04（UPG-97 合 main 随批裁决转立；产品决策项非缺陷）</t>
         </is>
       </c>
-      <c r="H89" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I89" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-    </row>
-    <row r="90">
-      <c r="A90" t="inlineStr">
+      <c r="H98" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I98" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
         <is>
           <t>UPG-102</t>
         </is>
       </c>
-      <c r="B90" t="inlineStr">
+      <c r="B99" t="inlineStr">
         <is>
           <t>MainActivity 拆分·批③ 页面桥面搬移（→ pages/ 模块）</t>
         </is>
       </c>
-      <c r="C90" t="inlineStr">
+      <c r="C99" t="inlineStr">
         <is>
           <t>P1 → ✅ **验收员复验 通过 @2026-09-04**（ACCEPTANCE_LOG §P53：**真交付=d77dae2a**[申报 cfa7d607 错误——申报 sha 错误 P3]隔离 worktree——全量 **809/0/1 亲跑一致**+PagesSplitContractTest 5 用例[申报 6 差 1 注记]+**M2 亲杀**[browser.forward 行置空→「漏搬 browser handler」红→还原]+approvalService internal 复核；两块搬移纯搬移核物；**达待合→审验员→设计师**）
 → 🆕 **已认领 @2026-09-04**（程序员 Claude/wmw0027，worktree mov-upg102，branch feat/upg102，基 main d11509cc；施工：browserHandlers 注册块[14 个 browser.*]+WebMcpHub.mountCallback 块→pages/ 模块顶层扩展——纯搬移零逻辑改动+3 变异锚+锚定面迁移收口[全量 0 失败硬门槛]+搬出函数显式 internal）
@@ -4665,361 +5088,361 @@
 → **防撞**：本批独占 MainActivity 页面桥区；与在飞单零交集；批④</t>
         </is>
       </c>
-      <c r="D90" t="inlineStr">
+      <c r="D99" t="inlineStr">
         <is>
           <t>📌 **已派单·待认领 @2026-09-04**（拆分主线批③/共 8 批｜串行纪律：批② d11509cc 已合，本批基=main 顶</t>
         </is>
       </c>
-      <c r="E90" t="inlineStr">
+      <c r="E99" t="inlineStr">
         <is>
           <t>🆕 **已认领 @2026-09-04**（程序员 Claude/wmw0027，worktree mov-upg102，branch f</t>
         </is>
       </c>
-      <c r="F90" t="inlineStr">
+      <c r="F99" t="inlineStr">
         <is>
           <t>✅ **审验员独立复核 通过 @2026-09-04**（§P53 审验终态：从零编译 809/0/0+1 跳过 + 契约锚 5/5 + M</t>
         </is>
       </c>
-      <c r="G90" t="inlineStr">
+      <c r="G99" t="inlineStr">
         <is>
           <t>✅ **已合 main @cfa7d607（2026-09-04 设计师合入：fast-forward d11509cc→cfa7d607</t>
         </is>
       </c>
-      <c r="H90" t="inlineStr">
+      <c r="H99" t="inlineStr">
         <is>
           <t>设计师\派单\UPG-102_MainActivity拆分批3页面桥_派单_2026-09-04.md</t>
         </is>
       </c>
-      <c r="I90" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-    </row>
-    <row r="91">
-      <c r="A91" t="inlineStr">
+      <c r="I99" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
         <is>
           <t>UPG-103</t>
         </is>
       </c>
-      <c r="B91" t="inlineStr">
+      <c r="B100" t="inlineStr">
         <is>
           <t>MainActivity 拆分·批④ chips/胶囊面搬移（→ ui/chips/ + ui/capsule/）</t>
         </is>
       </c>
-      <c r="C91" t="inlineStr">
+      <c r="C100" t="inlineStr">
         <is>
           <t>P1 → 🆕 **已认领 @2026-09-04 20:50**</t>
         </is>
       </c>
-      <c r="D91" t="inlineStr">
+      <c r="D100" t="inlineStr">
         <is>
           <t>📌 **已派单·待认领 @2026-09-04**</t>
         </is>
       </c>
-      <c r="E91" t="inlineStr">
+      <c r="E100" t="inlineStr">
         <is>
           <t>✅ **C 交付 @2026-09-04 23:05**（feat/upg103 **4e5a2f7c** 已 push origin；设计</t>
         </is>
       </c>
-      <c r="F91" t="inlineStr">
+      <c r="F100" t="inlineStr">
         <is>
           <t>✅ **审验员转通过 @2026-09-05**（四断收口逐项复核全绿：STD v2 重冻=51584a7d 一致/DEL 绑定 manif</t>
         </is>
       </c>
-      <c r="G91" t="inlineStr">
+      <c r="G100" t="inlineStr">
         <is>
           <t>✅ **设计师合 main @97d7ca31**（2026-09-05：批④ chips/胶囊面搬移全链合入；合后 verify-hash</t>
         </is>
       </c>
-      <c r="H91" t="inlineStr">
+      <c r="H100" t="inlineStr">
         <is>
           <t>设计师\派单\UPG-103_MainActivity拆分批4芯片胶囊_派单_2026-09-04.md</t>
         </is>
       </c>
-      <c r="I91" t="inlineStr">
+      <c r="I100" t="inlineStr">
         <is>
           <t>DEL-UPG103-20260904-001</t>
         </is>
       </c>
     </row>
-    <row r="92">
-      <c r="A92" t="inlineStr">
+    <row r="101">
+      <c r="A101" t="inlineStr">
         <is>
           <t>UPG-104</t>
         </is>
       </c>
-      <c r="B92" t="inlineStr">
+      <c r="B101" t="inlineStr">
         <is>
           <t>工具联动 Runtime 契约·段②（评测集+安全门+编排+记忆回流）</t>
         </is>
       </c>
-      <c r="C92" t="inlineStr">
+      <c r="C101" t="inlineStr">
         <is>
           <t>P2</t>
         </is>
       </c>
-      <c r="D92" t="inlineStr">
+      <c r="D101" t="inlineStr">
         <is>
           <t>设计 v3/v3.1 全量保留归本单；待 UPG-46 段①</t>
         </is>
       </c>
-      <c r="E92" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F92" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G92" t="inlineStr">
+      <c r="E101" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F101" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G101" t="inlineStr">
         <is>
           <t>合 main后拆派单）</t>
         </is>
       </c>
-      <c r="H92" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I92" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-    </row>
-    <row r="93">
-      <c r="A93" t="inlineStr">
+      <c r="H101" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I101" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
         <is>
           <t>UPG-105</t>
         </is>
       </c>
-      <c r="B93" t="inlineStr">
+      <c r="B102" t="inlineStr">
         <is>
           <t>MOV 官网·容器面（给 AI 读）建设</t>
         </is>
       </c>
-      <c r="C93" t="inlineStr">
+      <c r="C102" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
-      <c r="D93" t="inlineStr">
+      <c r="D102" t="inlineStr">
         <is>
           <t>📌 **已立卡·待派 @2026-09-04**（设计 v3 定稿：`设计师/方案设计/工单方案/官网容器面_给AI看内容_设计_v3_2</t>
         </is>
       </c>
-      <c r="E93" t="inlineStr">
+      <c r="E102" t="inlineStr">
         <is>
           <t>✅**C 完成 @2026-09-04**（feat/upg105 **841f591d** 已 push origin，基 main c5</t>
         </is>
       </c>
-      <c r="F93" t="inlineStr">
+      <c r="F102" t="inlineStr">
         <is>
           <t>✅ **验收员复验 通过 @2026-09-04**（ACCEPTANCE_LOG §P55：841f591d 隔离 worktree｜全量</t>
         </is>
       </c>
-      <c r="G93" t="inlineStr">
+      <c r="G102" t="inlineStr">
         <is>
           <t>✅ **已合 main @2026-09-04**（设计师 ff `c5bb94af..841f591d` 已推 origin；批二即 UP</t>
         </is>
       </c>
-      <c r="H93" t="inlineStr">
+      <c r="H102" t="inlineStr">
         <is>
           <t>设计师/方案设计/工单方案/官网容器面_给AI看内容_设计_v3_2026-09-04.md</t>
         </is>
       </c>
-      <c r="I93" t="inlineStr">
+      <c r="I102" t="inlineStr">
         <is>
           <t>DEL-UPG105-20260904-001</t>
         </is>
       </c>
     </row>
-    <row r="94">
-      <c r="A94" t="inlineStr">
+    <row r="103">
+      <c r="A103" t="inlineStr">
         <is>
           <t>UPG-106</t>
         </is>
       </c>
-      <c r="B94" t="inlineStr">
+      <c r="B103" t="inlineStr">
         <is>
           <t>数字人体 V1（2D 全身部位图 + 健身挂点）</t>
         </is>
       </c>
-      <c r="C94" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D94" t="inlineStr">
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D103" t="inlineStr">
         <is>
           <t>✅ **大神评审通过 8.8/10（有条件）@2026-09-05 → v2.1 冻结稿已出**：`人体载体/数字人体_融入MOV架构_评审</t>
         </is>
       </c>
-      <c r="E94" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F94" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G94" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H94" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I94" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-    </row>
-    <row r="95">
-      <c r="A95" t="inlineStr">
+      <c r="E103" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F103" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G103" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H103" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I103" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
         <is>
           <t>UPG-107</t>
         </is>
       </c>
-      <c r="B95" t="inlineStr">
+      <c r="B104" t="inlineStr">
         <is>
           <t>Memory OS 类型化 payload（Semantic 池子结构化演进）</t>
         </is>
       </c>
-      <c r="C95" t="inlineStr">
+      <c r="C104" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
-      <c r="D95" t="inlineStr">
+      <c r="D104" t="inlineStr">
         <is>
           <t>裁决位]；DEL-UPG107-20260905-001[code=31640fc8/artifact=fc07ee63/manifest=</t>
         </is>
       </c>
-      <c r="E95" t="inlineStr">
+      <c r="E104" t="inlineStr">
         <is>
           <t>✅**C 完成 @2026-09-05**（feat/upg107 **31640fc8** 已 push origin[origin=gi</t>
         </is>
       </c>
-      <c r="F95" t="inlineStr">
+      <c r="F104" t="inlineStr">
         <is>
           <t>审验ok:true]/报告=程序员/交付报告/DELIVERY_UPG107_2026-09-05.md｜状态区投影锚+交付段详）</t>
         </is>
       </c>
-      <c r="G95" t="inlineStr">
+      <c r="G104" t="inlineStr">
         <is>
           <t>已合 main @31640fc8（ff-only；P 段数 56→56 无丢失；验收+审验全链闭环）</t>
         </is>
       </c>
-      <c r="H95" t="inlineStr">
+      <c r="H104" t="inlineStr">
         <is>
           <t>设计师/方案设计/04_记忆/Memory_OS_类型化payload_设计_v1_2026-09-05.md</t>
         </is>
       </c>
-      <c r="I95" t="inlineStr">
+      <c r="I104" t="inlineStr">
         <is>
           <t>DEL-UPG107-20260905-001</t>
         </is>
       </c>
     </row>
-    <row r="96">
-      <c r="A96" t="inlineStr">
+    <row r="105">
+      <c r="A105" t="inlineStr">
         <is>
           <t>UPG-108</t>
         </is>
       </c>
-      <c r="B96" t="inlineStr">
+      <c r="B105" t="inlineStr">
         <is>
           <t>手机即服务器·官网用户面（扫码配对 + 手机内容投影上站）</t>
         </is>
       </c>
-      <c r="C96" t="inlineStr">
+      <c r="C105" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
-      <c r="D96" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E96" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F96" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G96" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H96" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I96" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-    </row>
-    <row r="97">
-      <c r="A97" t="inlineStr">
+      <c r="D105" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E105" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F105" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G105" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H105" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I105" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
         <is>
           <t>UPG-109</t>
         </is>
       </c>
-      <c r="B97" t="inlineStr">
+      <c r="B106" t="inlineStr">
         <is>
           <t>第三方站 WebMCP 接入性扫描（agent 浏览器前置探测）</t>
         </is>
       </c>
-      <c r="C97" t="inlineStr">
+      <c r="C106" t="inlineStr">
         <is>
           <t>P2</t>
         </is>
       </c>
-      <c r="D97" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E97" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F97" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G97" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H97" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I97" t="inlineStr">
+      <c r="D106" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E106" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F106" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G106" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H106" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I106" t="inlineStr">
         <is>
           <t>—</t>
         </is>

</xml_diff>

<commit_message>
UPG-110 交付：DELIVERY_UPG110_2026-09-05.md（六工具活端点生产上线+三变异锚亲杀+生产同源对账零差异+curl 三连实证）+ manifest 审验 ok:true——feat/upg110 1df4a3e3 set-status delivered 待验收
</commit_message>
<xml_diff>
--- a/工单系统/工单表.xlsx
+++ b/工单系统/工单表.xlsx
@@ -446,7 +446,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I106"/>
+  <dimension ref="A1:I107"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5443,6 +5443,53 @@
         </is>
       </c>
       <c r="I106" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>UPG-110</t>
+        </is>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>官网容器面·批二 A 通道（MCP Streamable HTTP 活端点）</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="D107" t="inlineStr">
+        <is>
+          <t>已派单（批二 A 通道，STD-UPG-110-v1 已冻结 99b78881）</t>
+        </is>
+      </c>
+      <c r="E107" t="inlineStr">
+        <is>
+          <t>已交付</t>
+        </is>
+      </c>
+      <c r="F107" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G107" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H107" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I107" t="inlineStr">
         <is>
           <t>—</t>
         </is>

</xml_diff>

<commit_message>
UPG-104 派单：段②解锁出单（STD-UPG-104-v1 冻结 sha=e6d8a7f9+派单文四件 A1-A4）+卡面六处校正（104 phase merged→registered 系 backfill 误判、100 dev/inspector 同步§P62、111 四列补齐§P64+head e396fab3、109 designer 补派单信息、83/106/111 优先级可解析化）——sync --sync 重建后 CHECK_OK diff=0 解析警告清零
</commit_message>
<xml_diff>
--- a/工单系统/工单表.xlsx
+++ b/工单系统/工单表.xlsx
@@ -4152,7 +4152,8 @@
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>P1（作废留档）
+→ **依据**：用户实测</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
@@ -4991,17 +4992,17 @@
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>📌 已派单（用户直接外派）</t>
+          <t>📌 已派单（用户直接外派）+ STD 追认冻结 @2026-09-05（简式）</t>
         </is>
       </c>
       <c r="E97" t="inlineStr">
         <is>
-          <t>✅ C 完成 @2026-09-05（kimi-cli，a63b7088——锚②升级 count/match；待验收）</t>
+          <t>✅ C 完成 @2026-09-05（kimi-cli，a63b7088——锚②升级 count/match）</t>
         </is>
       </c>
       <c r="F97" t="inlineStr">
         <is>
-          <t>📌 已立卡·待派 ⏳ @2026-09-04（UPG-96 审验发现项①转正：contains 组合锚对单点破坏免疫）｜ 待派单</t>
+          <t>✅ 复验通过 @2026-09-05（§P62 双变异亲杀+3 连跑零 flaky；达待合→审验员）</t>
         </is>
       </c>
       <c r="G97" t="inlineStr">
@@ -5179,12 +5180,12 @@
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>P2</t>
+          <t>P2 → ✅ **段①解锁 @2026-09-05**</t>
         </is>
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>设计 v3/v3.1 全量保留归本单；待 UPG-46 段①</t>
+          <t>📌 已派单·待认领 @2026-09-05（段① UPG-46 已合 main @7ccf0446 解锁；STD-UPG-104-v1 冻</t>
         </is>
       </c>
       <c r="E101" t="inlineStr">
@@ -5199,12 +5200,12 @@
       </c>
       <c r="G101" t="inlineStr">
         <is>
-          <t>合 main后拆派单）</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H101" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>设计师/派单/UPG-104_工具联动段2_派单_2026-09-05.md</t>
         </is>
       </c>
       <c r="I101" t="inlineStr">
@@ -5273,7 +5274,7 @@
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>P1</t>
         </is>
       </c>
       <c r="D103" t="inlineStr">
@@ -5419,7 +5420,7 @@
       </c>
       <c r="D106" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>📌 已派单·待认领 @2026-09-05（派单 `设计师/派单/UPG-109_第三方站WebMCP扫描器_派单_2026-09-05.</t>
         </is>
       </c>
       <c r="E106" t="inlineStr">
@@ -5508,22 +5509,22 @@
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>P3</t>
         </is>
       </c>
       <c r="D108" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>📌 立卡 @2026-09-05（P3——UPG-100 A3 死角扫尾转办）</t>
         </is>
       </c>
       <c r="E108" t="inlineStr">
         <is>
-          <t>已交付</t>
+          <t>✅ C 完成 @2026-09-05（e396fab3——18 处弱锚升级+3 代表变异亲杀）</t>
         </is>
       </c>
       <c r="F108" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>✅ 复验通过 @2026-09-05（§P64 定向 16/0+9/0+双刀抽杀亲红；达待合→审验员）</t>
         </is>
       </c>
       <c r="G108" t="inlineStr">

</xml_diff>

<commit_message>
UPG-100 合 main @2886821d 登记：审验✅（integrity_review=confirmed·独立四态亲杀）+隔离全量 844/0/1+终态 verify-hash HASH_OK+P3×2 销项（manifest standard_id 重绑 96c6bce1+落点归处理中心，--manifest 复跑 ok:True）——审验员落档（审验状态行/STD 会签/问题区）随行；sync diff=0
</commit_message>
<xml_diff>
--- a/工单系统/工单表.xlsx
+++ b/工单系统/工单表.xlsx
@@ -4992,7 +4992,7 @@
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>📌 已派单（用户直接外派）+ STD 追认冻结 @2026-09-05（简式）</t>
+          <t>📌 已派单（用户直接外派）+ STD 追认冻结 @2026-09-05（简式，sha=96c6bce1 会签已补）</t>
         </is>
       </c>
       <c r="E97" t="inlineStr">
@@ -5002,12 +5002,12 @@
       </c>
       <c r="F97" t="inlineStr">
         <is>
-          <t>✅ 复验通过 @2026-09-05（§P62 双变异亲杀+3 连跑零 flaky；达待合→审验员）</t>
+          <t>✅ 复验 §P62 + 审验✅ @2026-09-05（独立四态亲杀+A3 18 处表+STD 重算一致——integrity_review</t>
         </is>
       </c>
       <c r="G97" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>✅ 已合 main @2886821d（隔离全量 844/0/1；终态 verify-hash HASH_OK；P3×2 随批处置——man</t>
         </is>
       </c>
       <c r="H97" t="inlineStr">

</xml_diff>

<commit_message>
UPG-108 阶段1 demo 交付登记：DEL-UPG-108-20260906-001（feat/upg108 @ d1d87aa1 已 push；L1 22/22+全量862/0/1+变异5刀+信令线上闭环+8389双地址实证+报告/manifest/evidence 落盘；库卡 delivered+表 sync）
</commit_message>
<xml_diff>
--- a/工单系统/工单表.xlsx
+++ b/工单系统/工单表.xlsx
@@ -5379,7 +5379,7 @@
       </c>
       <c r="E105" t="inlineStr">
         <is>
-          <t>已认领</t>
+          <t>阶段1 demo 交付：L1 22/22+全量862/0/1+变异5刀全红+信令线上全链curl闭环+8389双地址真机实证+部署mov-a</t>
         </is>
       </c>
       <c r="F105" t="inlineStr">
@@ -5399,7 +5399,7 @@
       </c>
       <c r="I105" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>DEL-UPG-108-20260906-001</t>
         </is>
       </c>
     </row>

</xml_diff>